<commit_message>
chore: update coach knowledge base, export script, and video analysis docs
</commit_message>
<xml_diff>
--- a/client/knowledge/0_coach_knowledge/table_tennis_action_knowledge_v2.xlsx
+++ b/client/knowledge/0_coach_knowledge/table_tennis_action_knowledge_v2.xlsx
@@ -18,7 +18,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="739">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="734">
   <si>
     <t>乒乓球技术知识填写模板</t>
   </si>
@@ -993,10 +993,10 @@
     <t>已从md提取</t>
   </si>
   <si>
-    <t>肘部向前架起作为发力支点</t>
-  </si>
-  <si>
-    <t>区别于普通拨球的关键</t>
+    <t>持拍手的肘部向前架起作为发力支点，球拍头指向腹部方向</t>
+  </si>
+  <si>
+    <t>区别于普通拨球和拉球的关键</t>
   </si>
   <si>
     <t>标记为uncertain</t>
@@ -1005,7 +1005,7 @@
     <t>negative</t>
   </si>
   <si>
-    <t>无明显手腕内扣，前臂直接向前弹击</t>
+    <t>持拍手的肘部没有向前支架出去；无明显手腕内扣，前臂直接向前弹击</t>
   </si>
   <si>
     <t>更像反手拨球或拉球</t>
@@ -1029,7 +1029,7 @@
     <t>侧前方视角更容易观察，看球拍是否"包着球走"</t>
   </si>
   <si>
-    <t>前臂以肘为轴向前弹出，挥拍幅度小</t>
+    <t>持拍手和球拍在台面以上，前臂以肘为轴向前向外弹出，挥拍幅度小</t>
   </si>
   <si>
     <t>区分反手拨球和反手拉球的核心线索</t>
@@ -1038,7 +1038,7 @@
     <t>降低置信度，不要强判为反手拨球</t>
   </si>
   <si>
-    <t>引拍明显更低且向上摩擦充分</t>
+    <t>持拍手和球拍明显低于球台面，引拍明显更低且向上摩擦充分</t>
   </si>
   <si>
     <t>更像反手拉球</t>
@@ -1059,13 +1059,10 @@
     <t>preparation</t>
   </si>
   <si>
-    <t>肘部固定在身体前方不动</t>
-  </si>
-  <si>
-    <t>拨球动作稳定性的标志</t>
-  </si>
-  <si>
-    <t>蹲腿、转腰、收胯，手随身体引拍至腹前偏下，顶肘、手腕放松内屈</t>
+    <t>肘部固定在身体前方不动，击球点比较早，球刚跳起来未到最高点便击球</t>
+  </si>
+  <si>
+    <t>拨球的击球时机</t>
   </si>
   <si>
     <t>反手拉球重心及引拍特征</t>
@@ -1074,7 +1071,10 @@
     <t>无法确认时降低置信度</t>
   </si>
   <si>
-    <t>以肘为轴，前臂快速向右前外挥动，手腕内屈转外展形成鞭打</t>
+    <t>蹲腿、收胯，重心下压，持拍手随身体和重心引拍至腹前偏下，此时球拍低于球台面；持拍手的肘尖向持拍手外侧撑起使小臂与地面基本保持平行，手腕放松内屈</t>
+  </si>
+  <si>
+    <t>蹬腿、顶胯，体会用腹部将持拍手和球拍向外顶出；以肘为轴，前臂快速向右前上挥动。</t>
   </si>
   <si>
     <t>反手拉球发力特征</t>
@@ -1086,7 +1086,7 @@
     <t>更像反手拨球</t>
   </si>
   <si>
-    <t>在下降期或最高点摩擦球中上部，向上向前制造强烈上旋</t>
+    <t>在下降期或最高点摩擦球中上部，向前上方制造强烈上旋</t>
   </si>
   <si>
     <t>拉球的关键触球特征</t>
@@ -1402,7 +1402,7 @@
 反手拉球要等球的过了最高点的下降前期及球的中部，人离球台稍远，击球节奏一般较慢，需要空间和时间蓄力发力。</t>
   </si>
   <si>
-    <t>引拍幅度、挥拍方向、触球阶段</t>
+    <t>引拍幅度、腿和重心起伏、挥拍方向、触球阶段</t>
   </si>
   <si>
     <t>同时输出top2候选，不进入强诊断</t>
@@ -1411,13 +1411,13 @@
     <t>如果引拍和触球方向不可见，不要在bh_drive与bh_loop间强判。</t>
   </si>
   <si>
-    <t>拧拉多处理台内短球，手腕内扣外展明显；拨球更偏近台出台球衔接</t>
-  </si>
-  <si>
-    <t>拧拉肘部支点更突出</t>
-  </si>
-  <si>
-    <t>球是否台内、手腕动作、肘部位置</t>
+    <t>拧拉多处理台内短球，持拍手和球拍在台内，持拍手胳膊肘明显向外向前支出；拨球更偏近台出台球衔接</t>
+  </si>
+  <si>
+    <t>拧拉：持拍手手腕内扣外展明显，球拍拍头指向腹部。</t>
+  </si>
+  <si>
+    <t>持拍手以及球拍是否在台内、手腕动作、肘部位置</t>
   </si>
   <si>
     <t>标记uncertain，要求更清晰侧前方视角</t>
@@ -1426,7 +1426,7 @@
     <t>看不到球台短长时，不要高置信度识别bh_flick。</t>
   </si>
   <si>
-    <t>攻球引拍极小、撞击为主；拉球引拍幅度大、蹬转充分、向上摩擦明显</t>
+    <t>正手攻球引拍极小、撞击为主；拉球引拍幅度大、蹬转充分、向上摩擦明显</t>
   </si>
   <si>
     <t>拉球收臂至眉心位置，攻球前臂快速收缩</t>
@@ -2282,21 +2282,6 @@
   </si>
   <si>
     <t>发力速度</t>
-  </si>
-  <si>
-    <t>bh_drive_intended_loop</t>
-  </si>
-  <si>
-    <t>引拍极小、没有蹲腿转腰蓄力，动作幅度偏小</t>
-  </si>
-  <si>
-    <t>动作幅度过小，像拨球（针对拉球练习者）</t>
-  </si>
-  <si>
-    <t>系统检测到当前的动作更偏向反手拨球。如果你当前的训练目标是『反手拉球』，请注意你的动作幅度太小了：需要增加下蹲蓄力，并加大向上摩擦的幅度，不要仅仅靠前臂去撞击球。</t>
-  </si>
-  <si>
-    <t>引拍幅度、蹲腿转腰</t>
   </si>
   <si>
     <t>脚本和下拉框使用的候选值。通常不需要教练修改。</t>
@@ -2421,7 +2406,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="50">
+  <borders count="48">
     <border>
       <left/>
       <right/>
@@ -3022,37 +3007,13 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color indexed="11"/>
-      </left>
-      <right/>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left/>
-      <right/>
-      <top style="thin">
-        <color indexed="11"/>
-      </top>
-      <bottom style="thin">
-        <color indexed="11"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="97">
+  <cellXfs count="99">
     <xf numFmtId="0" fontId="0" applyNumberFormat="0" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
@@ -3218,39 +3179,57 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="38" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="24" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="24" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="25" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="27" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="27" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="7" borderId="28" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="39" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="39" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="4" borderId="40" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="8" borderId="40" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="40" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="4" borderId="40" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="8" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="12" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
@@ -3263,13 +3242,13 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="41" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="4" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="8" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="9" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="8" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="5" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="4" borderId="11" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -3284,7 +3263,10 @@
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="9" borderId="21" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="20" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
+      <alignment vertical="bottom" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="8" borderId="22" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="0" fillId="7" borderId="23" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
@@ -3322,21 +3304,6 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="4" borderId="29" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom" wrapText="1"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="48" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="4" borderId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="49" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="49" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="4" borderId="38" applyNumberFormat="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="0">
-      <alignment vertical="bottom"/>
     </xf>
     <xf numFmtId="0" fontId="0" applyNumberFormat="1" applyFont="1" applyFill="0" applyBorder="0" applyAlignment="1" applyProtection="0">
       <alignment vertical="bottom"/>
@@ -3370,8 +3337,8 @@
       <rgbColor rgb="ff2f6b8f"/>
       <rgbColor rgb="ff729fb3"/>
       <rgbColor rgb="ffd0dfe5"/>
+      <rgbColor rgb="ffa6d396"/>
       <rgbColor rgb="ffffff00"/>
-      <rgbColor rgb="ffa6d396"/>
     </indexedColors>
   </colors>
 </styleSheet>
@@ -6106,7 +6073,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I58"/>
+  <dimension ref="A1:I59"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col min="1" max="1" width="14.5" style="53" customWidth="1"/>
@@ -6194,10 +6161,10 @@
       <c r="C5" t="s" s="32">
         <v>291</v>
       </c>
-      <c r="D5" t="s" s="32">
+      <c r="D5" t="s" s="55">
         <v>292</v>
       </c>
-      <c r="E5" s="55">
+      <c r="E5" s="56">
         <v>3</v>
       </c>
       <c r="F5" t="s" s="32">
@@ -6221,11 +6188,11 @@
       <c r="C6" t="s" s="35">
         <v>73</v>
       </c>
-      <c r="D6" t="s" s="35">
+      <c r="D6" t="s" s="57">
         <v>296</v>
       </c>
-      <c r="E6" s="56">
-        <v>2</v>
+      <c r="E6" s="58">
+        <v>3</v>
       </c>
       <c r="F6" t="s" s="35">
         <v>297</v>
@@ -6233,7 +6200,7 @@
       <c r="G6" t="s" s="35">
         <v>298</v>
       </c>
-      <c r="H6" s="57"/>
+      <c r="H6" s="59"/>
       <c r="I6" s="29"/>
     </row>
     <row r="7" ht="31.5" customHeight="1">
@@ -6246,10 +6213,10 @@
       <c r="C7" t="s" s="38">
         <v>73</v>
       </c>
-      <c r="D7" t="s" s="38">
+      <c r="D7" t="s" s="60">
         <v>300</v>
       </c>
-      <c r="E7" s="58">
+      <c r="E7" s="61">
         <v>3</v>
       </c>
       <c r="F7" t="s" s="38">
@@ -6258,1353 +6225,1378 @@
       <c r="G7" t="s" s="38">
         <v>302</v>
       </c>
-      <c r="H7" s="59"/>
+      <c r="H7" s="62"/>
       <c r="I7" s="29"/>
     </row>
     <row r="8" ht="31.5" customHeight="1">
-      <c r="A8" t="s" s="60">
+      <c r="A8" t="s" s="63">
         <v>125</v>
       </c>
-      <c r="B8" t="s" s="61">
+      <c r="B8" t="s" s="64">
         <v>70</v>
       </c>
-      <c r="C8" t="s" s="61">
+      <c r="C8" t="s" s="64">
         <v>303</v>
       </c>
-      <c r="D8" t="s" s="61">
+      <c r="D8" t="s" s="65">
         <v>304</v>
       </c>
-      <c r="E8" s="62">
+      <c r="E8" s="66">
         <v>2</v>
       </c>
-      <c r="F8" t="s" s="61">
+      <c r="F8" t="s" s="64">
         <v>305</v>
       </c>
-      <c r="G8" t="s" s="61">
+      <c r="G8" t="s" s="64">
         <v>306</v>
       </c>
-      <c r="H8" t="s" s="61">
+      <c r="H8" t="s" s="64">
         <v>307</v>
       </c>
       <c r="I8" s="54"/>
     </row>
-    <row r="9" ht="31.5" customHeight="1">
-      <c r="A9" t="s" s="63">
+    <row r="9" ht="35" customHeight="1">
+      <c r="A9" t="s" s="67">
         <v>33</v>
       </c>
-      <c r="B9" t="s" s="63">
+      <c r="B9" t="s" s="67">
         <v>70</v>
       </c>
-      <c r="C9" t="s" s="63">
+      <c r="C9" t="s" s="67">
         <v>303</v>
       </c>
-      <c r="D9" t="s" s="63">
+      <c r="D9" t="s" s="68">
         <v>308</v>
       </c>
-      <c r="E9" s="64">
+      <c r="E9" s="69">
         <v>3</v>
       </c>
-      <c r="F9" t="s" s="63">
+      <c r="F9" t="s" s="67">
         <v>309</v>
       </c>
-      <c r="G9" t="s" s="63">
+      <c r="G9" t="s" s="67">
         <v>310</v>
       </c>
-      <c r="H9" t="s" s="63">
+      <c r="H9" t="s" s="67">
         <v>20</v>
       </c>
       <c r="I9" s="30"/>
     </row>
     <row r="10" ht="31.5" customHeight="1">
-      <c r="A10" t="s" s="65">
+      <c r="A10" t="s" s="70">
         <v>33</v>
       </c>
-      <c r="B10" t="s" s="65">
+      <c r="B10" t="s" s="70">
         <v>299</v>
       </c>
-      <c r="C10" t="s" s="65">
+      <c r="C10" t="s" s="70">
         <v>73</v>
       </c>
-      <c r="D10" t="s" s="65">
+      <c r="D10" t="s" s="71">
         <v>311</v>
       </c>
-      <c r="E10" s="66">
+      <c r="E10" s="72">
         <v>3</v>
       </c>
-      <c r="F10" t="s" s="65">
+      <c r="F10" t="s" s="70">
         <v>312</v>
       </c>
-      <c r="G10" t="s" s="65">
+      <c r="G10" t="s" s="70">
         <v>313</v>
       </c>
-      <c r="H10" t="s" s="65">
+      <c r="H10" t="s" s="70">
         <v>20</v>
       </c>
       <c r="I10" s="30"/>
     </row>
     <row r="11" ht="31.5" customHeight="1">
-      <c r="A11" t="s" s="65">
+      <c r="A11" t="s" s="70">
         <v>33</v>
       </c>
-      <c r="B11" t="s" s="65">
+      <c r="B11" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C11" t="s" s="65">
+      <c r="C11" t="s" s="70">
         <v>291</v>
       </c>
-      <c r="D11" t="s" s="65">
+      <c r="D11" t="s" s="71">
         <v>314</v>
       </c>
-      <c r="E11" s="66">
+      <c r="E11" s="72">
         <v>2</v>
       </c>
-      <c r="F11" t="s" s="65">
+      <c r="F11" t="s" s="70">
         <v>315</v>
       </c>
-      <c r="G11" t="s" s="65">
+      <c r="G11" t="s" s="70">
         <v>316</v>
       </c>
-      <c r="H11" t="s" s="65">
+      <c r="H11" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I11" s="30"/>
     </row>
     <row r="12" ht="31.5" customHeight="1">
-      <c r="A12" t="s" s="65">
+      <c r="A12" t="s" s="70">
         <v>33</v>
       </c>
-      <c r="B12" t="s" s="65">
+      <c r="B12" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C12" t="s" s="65">
+      <c r="C12" t="s" s="70">
         <v>317</v>
       </c>
-      <c r="D12" t="s" s="65">
+      <c r="D12" t="s" s="71">
         <v>318</v>
       </c>
-      <c r="E12" s="66">
+      <c r="E12" s="72">
+        <v>3</v>
+      </c>
+      <c r="F12" t="s" s="70">
+        <v>319</v>
+      </c>
+      <c r="G12" t="s" s="70">
+        <v>316</v>
+      </c>
+      <c r="H12" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I12" s="30"/>
+    </row>
+    <row r="13" ht="31.5" customHeight="1">
+      <c r="A13" t="s" s="70">
+        <v>97</v>
+      </c>
+      <c r="B13" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C13" t="s" s="70">
+        <v>73</v>
+      </c>
+      <c r="D13" t="s" s="71">
+        <v>311</v>
+      </c>
+      <c r="E13" s="72">
+        <v>3</v>
+      </c>
+      <c r="F13" t="s" s="70">
+        <v>320</v>
+      </c>
+      <c r="G13" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H13" s="70"/>
+      <c r="I13" s="30"/>
+    </row>
+    <row r="14" ht="67" customHeight="1">
+      <c r="A14" t="s" s="70">
+        <v>97</v>
+      </c>
+      <c r="B14" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C14" t="s" s="70">
+        <v>73</v>
+      </c>
+      <c r="D14" t="s" s="71">
+        <v>322</v>
+      </c>
+      <c r="E14" s="72">
+        <v>3</v>
+      </c>
+      <c r="F14" t="s" s="70">
+        <v>320</v>
+      </c>
+      <c r="G14" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H14" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I14" s="30"/>
+    </row>
+    <row r="15" ht="35" customHeight="1">
+      <c r="A15" t="s" s="70">
+        <v>97</v>
+      </c>
+      <c r="B15" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C15" t="s" s="70">
+        <v>303</v>
+      </c>
+      <c r="D15" t="s" s="71">
+        <v>323</v>
+      </c>
+      <c r="E15" s="72">
+        <v>3</v>
+      </c>
+      <c r="F15" t="s" s="70">
+        <v>324</v>
+      </c>
+      <c r="G15" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H15" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I15" s="30"/>
+    </row>
+    <row r="16" ht="31.5" customHeight="1">
+      <c r="A16" t="s" s="70">
+        <v>97</v>
+      </c>
+      <c r="B16" t="s" s="70">
+        <v>299</v>
+      </c>
+      <c r="C16" t="s" s="70">
+        <v>303</v>
+      </c>
+      <c r="D16" t="s" s="71">
+        <v>325</v>
+      </c>
+      <c r="E16" s="72">
+        <v>3</v>
+      </c>
+      <c r="F16" t="s" s="70">
+        <v>326</v>
+      </c>
+      <c r="G16" t="s" s="70">
+        <v>302</v>
+      </c>
+      <c r="H16" s="30"/>
+      <c r="I16" s="30"/>
+    </row>
+    <row r="17" ht="35" customHeight="1">
+      <c r="A17" t="s" s="70">
+        <v>97</v>
+      </c>
+      <c r="B17" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C17" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D17" t="s" s="71">
+        <v>327</v>
+      </c>
+      <c r="E17" s="72">
         <v>2</v>
       </c>
-      <c r="F12" t="s" s="65">
-        <v>319</v>
-      </c>
-      <c r="G12" t="s" s="65">
+      <c r="F17" t="s" s="70">
+        <v>328</v>
+      </c>
+      <c r="G17" t="s" s="70">
         <v>316</v>
       </c>
-      <c r="H12" t="s" s="65">
+      <c r="H17" t="s" s="70">
         <v>295</v>
       </c>
-      <c r="I12" s="30"/>
-    </row>
-    <row r="13" ht="31.5" customHeight="1">
-      <c r="A13" t="s" s="65">
-        <v>97</v>
-      </c>
-      <c r="B13" t="s" s="65">
+      <c r="I17" s="30"/>
+    </row>
+    <row r="18" ht="31.5" customHeight="1">
+      <c r="A18" t="s" s="70">
+        <v>207</v>
+      </c>
+      <c r="B18" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C13" t="s" s="65">
+      <c r="C18" t="s" s="70">
+        <v>317</v>
+      </c>
+      <c r="D18" t="s" s="70">
+        <v>329</v>
+      </c>
+      <c r="E18" s="72">
+        <v>3</v>
+      </c>
+      <c r="F18" t="s" s="70">
+        <v>330</v>
+      </c>
+      <c r="G18" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H18" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I18" s="30"/>
+    </row>
+    <row r="19" ht="31.5" customHeight="1">
+      <c r="A19" t="s" s="70">
+        <v>207</v>
+      </c>
+      <c r="B19" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C19" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D19" t="s" s="70">
+        <v>331</v>
+      </c>
+      <c r="E19" s="72">
+        <v>3</v>
+      </c>
+      <c r="F19" t="s" s="70">
+        <v>332</v>
+      </c>
+      <c r="G19" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H19" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I19" s="30"/>
+    </row>
+    <row r="20" ht="31.5" customHeight="1">
+      <c r="A20" t="s" s="70">
+        <v>207</v>
+      </c>
+      <c r="B20" t="s" s="70">
+        <v>299</v>
+      </c>
+      <c r="C20" t="s" s="70">
         <v>73</v>
       </c>
-      <c r="D13" t="s" s="65">
-        <v>320</v>
-      </c>
-      <c r="E13" s="66">
+      <c r="D20" t="s" s="70">
+        <v>333</v>
+      </c>
+      <c r="E20" s="72">
+        <v>2</v>
+      </c>
+      <c r="F20" t="s" s="70">
+        <v>334</v>
+      </c>
+      <c r="G20" t="s" s="70">
+        <v>335</v>
+      </c>
+      <c r="H20" s="30"/>
+      <c r="I20" s="30"/>
+    </row>
+    <row r="21" ht="31.5" customHeight="1">
+      <c r="A21" t="s" s="70">
+        <v>207</v>
+      </c>
+      <c r="B21" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C21" t="s" s="70">
+        <v>336</v>
+      </c>
+      <c r="D21" t="s" s="70">
+        <v>337</v>
+      </c>
+      <c r="E21" s="72">
+        <v>1</v>
+      </c>
+      <c r="F21" t="s" s="70">
+        <v>338</v>
+      </c>
+      <c r="G21" t="s" s="70">
+        <v>316</v>
+      </c>
+      <c r="H21" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I21" s="30"/>
+    </row>
+    <row r="22" ht="31.5" customHeight="1">
+      <c r="A22" t="s" s="70">
+        <v>215</v>
+      </c>
+      <c r="B22" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C22" t="s" s="70">
+        <v>73</v>
+      </c>
+      <c r="D22" t="s" s="70">
+        <v>339</v>
+      </c>
+      <c r="E22" s="72">
         <v>3</v>
       </c>
-      <c r="F13" t="s" s="65">
+      <c r="F22" t="s" s="70">
+        <v>340</v>
+      </c>
+      <c r="G22" t="s" s="70">
         <v>321</v>
       </c>
-      <c r="G13" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H13" t="s" s="65">
+      <c r="H22" t="s" s="70">
         <v>295</v>
       </c>
-      <c r="I13" s="30"/>
-    </row>
-    <row r="14" ht="31.5" customHeight="1">
-      <c r="A14" t="s" s="65">
-        <v>97</v>
-      </c>
-      <c r="B14" t="s" s="65">
+      <c r="I22" s="30"/>
+    </row>
+    <row r="23" ht="31.5" customHeight="1">
+      <c r="A23" t="s" s="70">
+        <v>215</v>
+      </c>
+      <c r="B23" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C14" t="s" s="65">
+      <c r="C23" t="s" s="70">
         <v>303</v>
       </c>
-      <c r="D14" t="s" s="65">
-        <v>323</v>
-      </c>
-      <c r="E14" s="66">
+      <c r="D23" t="s" s="70">
+        <v>341</v>
+      </c>
+      <c r="E23" s="72">
         <v>3</v>
       </c>
-      <c r="F14" t="s" s="65">
-        <v>324</v>
-      </c>
-      <c r="G14" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H14" t="s" s="65">
+      <c r="F23" t="s" s="70">
+        <v>342</v>
+      </c>
+      <c r="G23" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H23" t="s" s="70">
         <v>295</v>
       </c>
-      <c r="I14" s="30"/>
-    </row>
-    <row r="15" ht="31.5" customHeight="1">
-      <c r="A15" t="s" s="65">
-        <v>97</v>
-      </c>
-      <c r="B15" t="s" s="65">
+      <c r="I23" s="30"/>
+    </row>
+    <row r="24" ht="31.5" customHeight="1">
+      <c r="A24" t="s" s="70">
+        <v>215</v>
+      </c>
+      <c r="B24" t="s" s="70">
         <v>299</v>
       </c>
-      <c r="C15" t="s" s="65">
+      <c r="C24" t="s" s="70">
+        <v>73</v>
+      </c>
+      <c r="D24" t="s" s="70">
+        <v>343</v>
+      </c>
+      <c r="E24" s="72">
+        <v>3</v>
+      </c>
+      <c r="F24" t="s" s="70">
+        <v>344</v>
+      </c>
+      <c r="G24" t="s" s="70">
+        <v>345</v>
+      </c>
+      <c r="H24" s="30"/>
+      <c r="I24" s="30"/>
+    </row>
+    <row r="25" ht="31.5" customHeight="1">
+      <c r="A25" t="s" s="70">
+        <v>215</v>
+      </c>
+      <c r="B25" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C25" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D25" t="s" s="70">
+        <v>346</v>
+      </c>
+      <c r="E25" s="72">
+        <v>2</v>
+      </c>
+      <c r="F25" t="s" s="70">
+        <v>347</v>
+      </c>
+      <c r="G25" t="s" s="70">
+        <v>316</v>
+      </c>
+      <c r="H25" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I25" s="30"/>
+    </row>
+    <row r="26" ht="31.5" customHeight="1">
+      <c r="A26" t="s" s="70">
+        <v>149</v>
+      </c>
+      <c r="B26" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C26" t="s" s="70">
+        <v>73</v>
+      </c>
+      <c r="D26" t="s" s="70">
+        <v>348</v>
+      </c>
+      <c r="E26" s="72">
+        <v>3</v>
+      </c>
+      <c r="F26" t="s" s="70">
+        <v>349</v>
+      </c>
+      <c r="G26" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H26" t="s" s="70">
+        <v>20</v>
+      </c>
+      <c r="I26" s="30"/>
+    </row>
+    <row r="27" ht="31.5" customHeight="1">
+      <c r="A27" t="s" s="70">
+        <v>149</v>
+      </c>
+      <c r="B27" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C27" t="s" s="70">
         <v>303</v>
       </c>
-      <c r="D15" t="s" s="65">
-        <v>325</v>
-      </c>
-      <c r="E15" s="66">
+      <c r="D27" t="s" s="70">
+        <v>350</v>
+      </c>
+      <c r="E27" s="72">
         <v>3</v>
       </c>
-      <c r="F15" t="s" s="65">
-        <v>326</v>
-      </c>
-      <c r="G15" t="s" s="65">
-        <v>302</v>
-      </c>
-      <c r="H15" s="30"/>
-      <c r="I15" s="30"/>
-    </row>
-    <row r="16" ht="31.5" customHeight="1">
-      <c r="A16" t="s" s="65">
-        <v>97</v>
-      </c>
-      <c r="B16" t="s" s="65">
+      <c r="F27" t="s" s="70">
+        <v>351</v>
+      </c>
+      <c r="G27" t="s" s="70">
+        <v>352</v>
+      </c>
+      <c r="H27" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I27" s="30"/>
+    </row>
+    <row r="28" ht="31.5" customHeight="1">
+      <c r="A28" t="s" s="70">
+        <v>149</v>
+      </c>
+      <c r="B28" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C16" t="s" s="65">
+      <c r="C28" t="s" s="70">
         <v>291</v>
       </c>
-      <c r="D16" t="s" s="65">
-        <v>327</v>
-      </c>
-      <c r="E16" s="66">
+      <c r="D28" t="s" s="70">
+        <v>353</v>
+      </c>
+      <c r="E28" s="72">
         <v>2</v>
       </c>
-      <c r="F16" t="s" s="65">
-        <v>328</v>
-      </c>
-      <c r="G16" t="s" s="65">
+      <c r="F28" t="s" s="70">
+        <v>354</v>
+      </c>
+      <c r="G28" t="s" s="70">
         <v>316</v>
       </c>
-      <c r="H16" t="s" s="65">
+      <c r="H28" t="s" s="70">
         <v>295</v>
       </c>
-      <c r="I16" s="30"/>
-    </row>
-    <row r="17" ht="31.5" customHeight="1">
-      <c r="A17" t="s" s="65">
-        <v>207</v>
-      </c>
-      <c r="B17" t="s" s="65">
+      <c r="I28" s="30"/>
+    </row>
+    <row r="29" ht="31.5" customHeight="1">
+      <c r="A29" t="s" s="70">
+        <v>149</v>
+      </c>
+      <c r="B29" t="s" s="70">
+        <v>299</v>
+      </c>
+      <c r="C29" t="s" s="70">
+        <v>303</v>
+      </c>
+      <c r="D29" t="s" s="70">
+        <v>355</v>
+      </c>
+      <c r="E29" s="72">
+        <v>3</v>
+      </c>
+      <c r="F29" t="s" s="70">
+        <v>356</v>
+      </c>
+      <c r="G29" t="s" s="70">
+        <v>357</v>
+      </c>
+      <c r="H29" s="30"/>
+      <c r="I29" s="30"/>
+    </row>
+    <row r="30" ht="31.5" customHeight="1">
+      <c r="A30" t="s" s="70">
+        <v>231</v>
+      </c>
+      <c r="B30" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C17" t="s" s="65">
+      <c r="C30" t="s" s="70">
         <v>317</v>
       </c>
-      <c r="D17" t="s" s="65">
-        <v>329</v>
-      </c>
-      <c r="E17" s="66">
+      <c r="D30" t="s" s="70">
+        <v>358</v>
+      </c>
+      <c r="E30" s="72">
         <v>3</v>
       </c>
-      <c r="F17" t="s" s="65">
-        <v>330</v>
-      </c>
-      <c r="G17" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H17" t="s" s="65">
+      <c r="F30" t="s" s="70">
+        <v>359</v>
+      </c>
+      <c r="G30" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H30" t="s" s="70">
         <v>295</v>
       </c>
-      <c r="I17" s="30"/>
-    </row>
-    <row r="18" ht="31.5" customHeight="1">
-      <c r="A18" t="s" s="65">
-        <v>207</v>
-      </c>
-      <c r="B18" t="s" s="65">
+      <c r="I30" s="30"/>
+    </row>
+    <row r="31" ht="31.5" customHeight="1">
+      <c r="A31" t="s" s="70">
+        <v>231</v>
+      </c>
+      <c r="B31" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C18" t="s" s="65">
+      <c r="C31" t="s" s="70">
         <v>291</v>
       </c>
-      <c r="D18" t="s" s="65">
-        <v>331</v>
-      </c>
-      <c r="E18" s="66">
+      <c r="D31" t="s" s="70">
+        <v>360</v>
+      </c>
+      <c r="E31" s="72">
         <v>3</v>
       </c>
-      <c r="F18" t="s" s="65">
-        <v>332</v>
-      </c>
-      <c r="G18" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H18" t="s" s="65">
+      <c r="F31" t="s" s="70">
+        <v>361</v>
+      </c>
+      <c r="G31" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H31" t="s" s="70">
         <v>295</v>
       </c>
-      <c r="I18" s="30"/>
-    </row>
-    <row r="19" ht="31.5" customHeight="1">
-      <c r="A19" t="s" s="65">
-        <v>207</v>
-      </c>
-      <c r="B19" t="s" s="65">
+      <c r="I31" s="30"/>
+    </row>
+    <row r="32" ht="31.5" customHeight="1">
+      <c r="A32" t="s" s="70">
+        <v>231</v>
+      </c>
+      <c r="B32" t="s" s="70">
         <v>299</v>
       </c>
-      <c r="C19" t="s" s="65">
+      <c r="C32" t="s" s="70">
         <v>73</v>
       </c>
-      <c r="D19" t="s" s="65">
-        <v>333</v>
-      </c>
-      <c r="E19" s="66">
+      <c r="D32" t="s" s="70">
+        <v>362</v>
+      </c>
+      <c r="E32" s="72">
         <v>2</v>
       </c>
-      <c r="F19" t="s" s="65">
-        <v>334</v>
-      </c>
-      <c r="G19" t="s" s="65">
-        <v>335</v>
-      </c>
-      <c r="H19" s="30"/>
-      <c r="I19" s="30"/>
-    </row>
-    <row r="20" ht="31.5" customHeight="1">
-      <c r="A20" t="s" s="65">
-        <v>207</v>
-      </c>
-      <c r="B20" t="s" s="65">
+      <c r="F32" t="s" s="70">
+        <v>363</v>
+      </c>
+      <c r="G32" t="s" s="70">
+        <v>364</v>
+      </c>
+      <c r="H32" s="30"/>
+      <c r="I32" s="30"/>
+    </row>
+    <row r="33" ht="31.5" customHeight="1">
+      <c r="A33" t="s" s="70">
+        <v>231</v>
+      </c>
+      <c r="B33" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C20" t="s" s="65">
+      <c r="C33" t="s" s="70">
         <v>336</v>
       </c>
-      <c r="D20" t="s" s="65">
-        <v>337</v>
-      </c>
-      <c r="E20" s="66">
+      <c r="D33" t="s" s="70">
+        <v>365</v>
+      </c>
+      <c r="E33" s="72">
         <v>1</v>
       </c>
-      <c r="F20" t="s" s="65">
-        <v>338</v>
-      </c>
-      <c r="G20" t="s" s="65">
+      <c r="F33" t="s" s="70">
+        <v>366</v>
+      </c>
+      <c r="G33" t="s" s="70">
         <v>316</v>
       </c>
-      <c r="H20" t="s" s="65">
+      <c r="H33" t="s" s="70">
         <v>295</v>
       </c>
-      <c r="I20" s="30"/>
-    </row>
-    <row r="21" ht="31.5" customHeight="1">
-      <c r="A21" t="s" s="65">
-        <v>215</v>
-      </c>
-      <c r="B21" t="s" s="65">
+      <c r="I33" s="30"/>
+    </row>
+    <row r="34" ht="31.5" customHeight="1">
+      <c r="A34" t="s" s="70">
+        <v>239</v>
+      </c>
+      <c r="B34" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C21" t="s" s="65">
+      <c r="C34" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D34" t="s" s="70">
+        <v>367</v>
+      </c>
+      <c r="E34" s="72">
+        <v>3</v>
+      </c>
+      <c r="F34" t="s" s="70">
+        <v>368</v>
+      </c>
+      <c r="G34" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H34" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I34" s="30"/>
+    </row>
+    <row r="35" ht="31.5" customHeight="1">
+      <c r="A35" t="s" s="70">
+        <v>239</v>
+      </c>
+      <c r="B35" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C35" t="s" s="70">
+        <v>317</v>
+      </c>
+      <c r="D35" t="s" s="70">
+        <v>369</v>
+      </c>
+      <c r="E35" s="72">
+        <v>2</v>
+      </c>
+      <c r="F35" t="s" s="70">
+        <v>370</v>
+      </c>
+      <c r="G35" t="s" s="70">
+        <v>316</v>
+      </c>
+      <c r="H35" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I35" s="30"/>
+    </row>
+    <row r="36" ht="31.5" customHeight="1">
+      <c r="A36" t="s" s="73">
+        <v>239</v>
+      </c>
+      <c r="B36" t="s" s="73">
+        <v>299</v>
+      </c>
+      <c r="C36" t="s" s="73">
+        <v>291</v>
+      </c>
+      <c r="D36" t="s" s="73">
+        <v>371</v>
+      </c>
+      <c r="E36" s="74">
+        <v>3</v>
+      </c>
+      <c r="F36" t="s" s="73">
+        <v>372</v>
+      </c>
+      <c r="G36" t="s" s="73">
+        <v>373</v>
+      </c>
+      <c r="H36" s="75"/>
+      <c r="I36" s="30"/>
+    </row>
+    <row r="37" ht="31.5" customHeight="1">
+      <c r="A37" t="s" s="76">
+        <v>239</v>
+      </c>
+      <c r="B37" t="s" s="77">
+        <v>70</v>
+      </c>
+      <c r="C37" t="s" s="77">
+        <v>374</v>
+      </c>
+      <c r="D37" t="s" s="77">
+        <v>375</v>
+      </c>
+      <c r="E37" s="78">
+        <v>1</v>
+      </c>
+      <c r="F37" t="s" s="77">
+        <v>376</v>
+      </c>
+      <c r="G37" t="s" s="77">
+        <v>377</v>
+      </c>
+      <c r="H37" t="s" s="77">
+        <v>378</v>
+      </c>
+      <c r="I37" s="54"/>
+    </row>
+    <row r="38" ht="31.5" customHeight="1">
+      <c r="A38" t="s" s="67">
+        <v>247</v>
+      </c>
+      <c r="B38" t="s" s="67">
+        <v>70</v>
+      </c>
+      <c r="C38" t="s" s="67">
         <v>73</v>
       </c>
-      <c r="D21" t="s" s="65">
-        <v>339</v>
-      </c>
-      <c r="E21" s="66">
+      <c r="D38" t="s" s="67">
+        <v>379</v>
+      </c>
+      <c r="E38" s="69">
         <v>3</v>
       </c>
-      <c r="F21" t="s" s="65">
-        <v>340</v>
-      </c>
-      <c r="G21" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H21" t="s" s="65">
+      <c r="F38" t="s" s="67">
+        <v>380</v>
+      </c>
+      <c r="G38" t="s" s="67">
+        <v>321</v>
+      </c>
+      <c r="H38" t="s" s="67">
         <v>295</v>
       </c>
-      <c r="I21" s="30"/>
-    </row>
-    <row r="22" ht="31.5" customHeight="1">
-      <c r="A22" t="s" s="65">
-        <v>215</v>
-      </c>
-      <c r="B22" t="s" s="65">
+      <c r="I38" s="30"/>
+    </row>
+    <row r="39" ht="31.5" customHeight="1">
+      <c r="A39" t="s" s="70">
+        <v>247</v>
+      </c>
+      <c r="B39" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C22" t="s" s="65">
+      <c r="C39" t="s" s="70">
         <v>303</v>
       </c>
-      <c r="D22" t="s" s="65">
-        <v>341</v>
-      </c>
-      <c r="E22" s="66">
+      <c r="D39" t="s" s="70">
+        <v>381</v>
+      </c>
+      <c r="E39" s="72">
         <v>3</v>
       </c>
-      <c r="F22" t="s" s="65">
-        <v>342</v>
-      </c>
-      <c r="G22" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H22" t="s" s="65">
+      <c r="F39" t="s" s="70">
+        <v>382</v>
+      </c>
+      <c r="G39" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H39" t="s" s="70">
         <v>295</v>
       </c>
-      <c r="I22" s="30"/>
-    </row>
-    <row r="23" ht="31.5" customHeight="1">
-      <c r="A23" t="s" s="65">
-        <v>215</v>
-      </c>
-      <c r="B23" t="s" s="65">
+      <c r="I39" s="30"/>
+    </row>
+    <row r="40" ht="31.5" customHeight="1">
+      <c r="A40" t="s" s="70">
+        <v>247</v>
+      </c>
+      <c r="B40" t="s" s="70">
         <v>299</v>
       </c>
-      <c r="C23" t="s" s="65">
+      <c r="C40" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D40" t="s" s="70">
+        <v>383</v>
+      </c>
+      <c r="E40" s="72">
+        <v>3</v>
+      </c>
+      <c r="F40" t="s" s="70">
+        <v>384</v>
+      </c>
+      <c r="G40" t="s" s="70">
+        <v>385</v>
+      </c>
+      <c r="H40" s="30"/>
+      <c r="I40" s="30"/>
+    </row>
+    <row r="41" ht="31.5" customHeight="1">
+      <c r="A41" t="s" s="70">
+        <v>247</v>
+      </c>
+      <c r="B41" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C41" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D41" t="s" s="70">
+        <v>386</v>
+      </c>
+      <c r="E41" s="72">
+        <v>2</v>
+      </c>
+      <c r="F41" t="s" s="70">
+        <v>387</v>
+      </c>
+      <c r="G41" t="s" s="70">
+        <v>316</v>
+      </c>
+      <c r="H41" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I41" s="30"/>
+    </row>
+    <row r="42" ht="31.5" customHeight="1">
+      <c r="A42" t="s" s="70">
+        <v>255</v>
+      </c>
+      <c r="B42" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C42" t="s" s="70">
         <v>73</v>
       </c>
-      <c r="D23" t="s" s="65">
-        <v>343</v>
-      </c>
-      <c r="E23" s="66">
+      <c r="D42" t="s" s="70">
+        <v>388</v>
+      </c>
+      <c r="E42" s="72">
         <v>3</v>
       </c>
-      <c r="F23" t="s" s="65">
-        <v>344</v>
-      </c>
-      <c r="G23" t="s" s="65">
+      <c r="F42" t="s" s="70">
+        <v>389</v>
+      </c>
+      <c r="G42" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H42" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I42" s="30"/>
+    </row>
+    <row r="43" ht="31.5" customHeight="1">
+      <c r="A43" t="s" s="70">
+        <v>255</v>
+      </c>
+      <c r="B43" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C43" t="s" s="70">
+        <v>303</v>
+      </c>
+      <c r="D43" t="s" s="70">
+        <v>390</v>
+      </c>
+      <c r="E43" s="72">
+        <v>3</v>
+      </c>
+      <c r="F43" t="s" s="70">
+        <v>391</v>
+      </c>
+      <c r="G43" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H43" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I43" s="30"/>
+    </row>
+    <row r="44" ht="31.5" customHeight="1">
+      <c r="A44" t="s" s="70">
+        <v>255</v>
+      </c>
+      <c r="B44" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C44" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D44" t="s" s="70">
+        <v>392</v>
+      </c>
+      <c r="E44" s="72">
+        <v>2</v>
+      </c>
+      <c r="F44" t="s" s="70">
+        <v>393</v>
+      </c>
+      <c r="G44" t="s" s="70">
+        <v>316</v>
+      </c>
+      <c r="H44" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I44" s="30"/>
+    </row>
+    <row r="45" ht="31.5" customHeight="1">
+      <c r="A45" t="s" s="70">
+        <v>255</v>
+      </c>
+      <c r="B45" t="s" s="70">
+        <v>299</v>
+      </c>
+      <c r="C45" t="s" s="70">
+        <v>303</v>
+      </c>
+      <c r="D45" t="s" s="70">
+        <v>394</v>
+      </c>
+      <c r="E45" s="72">
+        <v>2</v>
+      </c>
+      <c r="F45" t="s" s="70">
+        <v>395</v>
+      </c>
+      <c r="G45" t="s" s="70">
+        <v>373</v>
+      </c>
+      <c r="H45" s="30"/>
+      <c r="I45" s="30"/>
+    </row>
+    <row r="46" ht="31.5" customHeight="1">
+      <c r="A46" t="s" s="70">
+        <v>263</v>
+      </c>
+      <c r="B46" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C46" t="s" s="70">
+        <v>317</v>
+      </c>
+      <c r="D46" t="s" s="70">
+        <v>396</v>
+      </c>
+      <c r="E46" s="72">
+        <v>3</v>
+      </c>
+      <c r="F46" t="s" s="70">
+        <v>397</v>
+      </c>
+      <c r="G46" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H46" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I46" s="30"/>
+    </row>
+    <row r="47" ht="31.5" customHeight="1">
+      <c r="A47" t="s" s="70">
+        <v>263</v>
+      </c>
+      <c r="B47" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C47" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D47" t="s" s="70">
+        <v>398</v>
+      </c>
+      <c r="E47" s="72">
+        <v>3</v>
+      </c>
+      <c r="F47" t="s" s="70">
+        <v>399</v>
+      </c>
+      <c r="G47" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H47" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I47" s="30"/>
+    </row>
+    <row r="48" ht="31.5" customHeight="1">
+      <c r="A48" t="s" s="70">
+        <v>263</v>
+      </c>
+      <c r="B48" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C48" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D48" t="s" s="70">
+        <v>400</v>
+      </c>
+      <c r="E48" s="72">
+        <v>3</v>
+      </c>
+      <c r="F48" t="s" s="70">
+        <v>401</v>
+      </c>
+      <c r="G48" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H48" t="s" s="70">
+        <v>295</v>
+      </c>
+      <c r="I48" s="30"/>
+    </row>
+    <row r="49" ht="31.5" customHeight="1">
+      <c r="A49" t="s" s="70">
+        <v>263</v>
+      </c>
+      <c r="B49" t="s" s="70">
+        <v>299</v>
+      </c>
+      <c r="C49" t="s" s="70">
+        <v>303</v>
+      </c>
+      <c r="D49" t="s" s="70">
+        <v>402</v>
+      </c>
+      <c r="E49" s="72">
+        <v>2</v>
+      </c>
+      <c r="F49" t="s" s="70">
+        <v>403</v>
+      </c>
+      <c r="G49" t="s" s="70">
+        <v>404</v>
+      </c>
+      <c r="H49" s="30"/>
+      <c r="I49" s="30"/>
+    </row>
+    <row r="50" ht="31.5" customHeight="1">
+      <c r="A50" t="s" s="79">
+        <v>271</v>
+      </c>
+      <c r="B50" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C50" t="s" s="70">
+        <v>317</v>
+      </c>
+      <c r="D50" t="s" s="70">
+        <v>405</v>
+      </c>
+      <c r="E50" s="72">
+        <v>3</v>
+      </c>
+      <c r="F50" t="s" s="70">
+        <v>406</v>
+      </c>
+      <c r="G50" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H50" s="80"/>
+      <c r="I50" s="29"/>
+    </row>
+    <row r="51" ht="31.5" customHeight="1">
+      <c r="A51" t="s" s="79">
+        <v>271</v>
+      </c>
+      <c r="B51" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C51" t="s" s="70">
+        <v>303</v>
+      </c>
+      <c r="D51" t="s" s="70">
+        <v>407</v>
+      </c>
+      <c r="E51" s="72">
+        <v>3</v>
+      </c>
+      <c r="F51" t="s" s="70">
+        <v>408</v>
+      </c>
+      <c r="G51" t="s" s="70">
+        <v>321</v>
+      </c>
+      <c r="H51" s="80"/>
+      <c r="I51" s="29"/>
+    </row>
+    <row r="52" ht="31.5" customHeight="1">
+      <c r="A52" t="s" s="79">
+        <v>271</v>
+      </c>
+      <c r="B52" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C52" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D52" t="s" s="70">
+        <v>409</v>
+      </c>
+      <c r="E52" s="72">
+        <v>2</v>
+      </c>
+      <c r="F52" t="s" s="70">
+        <v>410</v>
+      </c>
+      <c r="G52" t="s" s="70">
+        <v>316</v>
+      </c>
+      <c r="H52" s="80"/>
+      <c r="I52" s="29"/>
+    </row>
+    <row r="53" ht="31.5" customHeight="1">
+      <c r="A53" t="s" s="79">
+        <v>271</v>
+      </c>
+      <c r="B53" t="s" s="70">
+        <v>299</v>
+      </c>
+      <c r="C53" t="s" s="70">
+        <v>73</v>
+      </c>
+      <c r="D53" t="s" s="70">
+        <v>411</v>
+      </c>
+      <c r="E53" s="72">
+        <v>3</v>
+      </c>
+      <c r="F53" t="s" s="70">
+        <v>412</v>
+      </c>
+      <c r="G53" t="s" s="70">
         <v>345</v>
       </c>
-      <c r="H23" s="30"/>
-      <c r="I23" s="30"/>
-    </row>
-    <row r="24" ht="31.5" customHeight="1">
-      <c r="A24" t="s" s="65">
-        <v>215</v>
-      </c>
-      <c r="B24" t="s" s="65">
+      <c r="H53" s="80"/>
+      <c r="I53" s="29"/>
+    </row>
+    <row r="54" ht="31.5" customHeight="1">
+      <c r="A54" t="s" s="79">
+        <v>271</v>
+      </c>
+      <c r="B54" t="s" s="70">
+        <v>299</v>
+      </c>
+      <c r="C54" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D54" t="s" s="70">
+        <v>413</v>
+      </c>
+      <c r="E54" s="72">
+        <v>2</v>
+      </c>
+      <c r="F54" t="s" s="70">
+        <v>414</v>
+      </c>
+      <c r="G54" t="s" s="70">
+        <v>404</v>
+      </c>
+      <c r="H54" s="80"/>
+      <c r="I54" s="29"/>
+    </row>
+    <row r="55" ht="31.5" customHeight="1">
+      <c r="A55" t="s" s="79">
+        <v>280</v>
+      </c>
+      <c r="B55" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C24" t="s" s="65">
+      <c r="C55" t="s" s="70">
         <v>291</v>
       </c>
-      <c r="D24" t="s" s="65">
-        <v>346</v>
-      </c>
-      <c r="E24" s="66">
+      <c r="D55" t="s" s="70">
+        <v>415</v>
+      </c>
+      <c r="E55" s="72">
+        <v>3</v>
+      </c>
+      <c r="F55" t="s" s="70">
+        <v>416</v>
+      </c>
+      <c r="G55" t="s" s="70">
+        <v>417</v>
+      </c>
+      <c r="H55" t="s" s="81">
+        <v>418</v>
+      </c>
+      <c r="I55" s="29"/>
+    </row>
+    <row r="56" ht="31.5" customHeight="1">
+      <c r="A56" t="s" s="79">
+        <v>280</v>
+      </c>
+      <c r="B56" t="s" s="70">
+        <v>70</v>
+      </c>
+      <c r="C56" t="s" s="70">
+        <v>317</v>
+      </c>
+      <c r="D56" t="s" s="70">
+        <v>419</v>
+      </c>
+      <c r="E56" s="72">
         <v>2</v>
       </c>
-      <c r="F24" t="s" s="65">
-        <v>347</v>
-      </c>
-      <c r="G24" t="s" s="65">
+      <c r="F56" t="s" s="70">
+        <v>420</v>
+      </c>
+      <c r="G56" t="s" s="70">
         <v>316</v>
       </c>
-      <c r="H24" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I24" s="30"/>
-    </row>
-    <row r="25" ht="31.5" customHeight="1">
-      <c r="A25" t="s" s="65">
-        <v>149</v>
-      </c>
-      <c r="B25" t="s" s="65">
+      <c r="H56" t="s" s="81">
+        <v>421</v>
+      </c>
+      <c r="I56" s="29"/>
+    </row>
+    <row r="57" ht="31.5" customHeight="1">
+      <c r="A57" t="s" s="79">
+        <v>280</v>
+      </c>
+      <c r="B57" t="s" s="70">
         <v>70</v>
       </c>
-      <c r="C25" t="s" s="65">
-        <v>73</v>
-      </c>
-      <c r="D25" t="s" s="65">
-        <v>348</v>
-      </c>
-      <c r="E25" s="66">
+      <c r="C57" t="s" s="70">
+        <v>422</v>
+      </c>
+      <c r="D57" t="s" s="70">
+        <v>423</v>
+      </c>
+      <c r="E57" s="72">
+        <v>2</v>
+      </c>
+      <c r="F57" t="s" s="70">
+        <v>424</v>
+      </c>
+      <c r="G57" t="s" s="70">
+        <v>316</v>
+      </c>
+      <c r="H57" s="80"/>
+      <c r="I57" s="29"/>
+    </row>
+    <row r="58" ht="31.5" customHeight="1">
+      <c r="A58" t="s" s="79">
+        <v>280</v>
+      </c>
+      <c r="B58" t="s" s="70">
+        <v>299</v>
+      </c>
+      <c r="C58" t="s" s="70">
+        <v>291</v>
+      </c>
+      <c r="D58" t="s" s="70">
+        <v>425</v>
+      </c>
+      <c r="E58" s="72">
         <v>3</v>
       </c>
-      <c r="F25" t="s" s="65">
-        <v>349</v>
-      </c>
-      <c r="G25" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H25" t="s" s="65">
-        <v>20</v>
-      </c>
-      <c r="I25" s="30"/>
-    </row>
-    <row r="26" ht="31.5" customHeight="1">
-      <c r="A26" t="s" s="65">
-        <v>149</v>
-      </c>
-      <c r="B26" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C26" t="s" s="65">
-        <v>303</v>
-      </c>
-      <c r="D26" t="s" s="65">
-        <v>350</v>
-      </c>
-      <c r="E26" s="66">
-        <v>3</v>
-      </c>
-      <c r="F26" t="s" s="65">
-        <v>351</v>
-      </c>
-      <c r="G26" t="s" s="65">
-        <v>352</v>
-      </c>
-      <c r="H26" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I26" s="30"/>
-    </row>
-    <row r="27" ht="31.5" customHeight="1">
-      <c r="A27" t="s" s="65">
-        <v>149</v>
-      </c>
-      <c r="B27" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C27" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D27" t="s" s="65">
-        <v>353</v>
-      </c>
-      <c r="E27" s="66">
+      <c r="F58" t="s" s="70">
+        <v>384</v>
+      </c>
+      <c r="G58" t="s" s="70">
+        <v>385</v>
+      </c>
+      <c r="H58" t="s" s="81">
+        <v>426</v>
+      </c>
+      <c r="I58" s="29"/>
+    </row>
+    <row r="59" ht="19" customHeight="1">
+      <c r="A59" t="s" s="79">
+        <v>280</v>
+      </c>
+      <c r="B59" t="s" s="70">
+        <v>299</v>
+      </c>
+      <c r="C59" t="s" s="70">
+        <v>422</v>
+      </c>
+      <c r="D59" t="s" s="70">
+        <v>427</v>
+      </c>
+      <c r="E59" s="72">
         <v>2</v>
       </c>
-      <c r="F27" t="s" s="65">
-        <v>354</v>
-      </c>
-      <c r="G27" t="s" s="65">
-        <v>316</v>
-      </c>
-      <c r="H27" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I27" s="30"/>
-    </row>
-    <row r="28" ht="31.5" customHeight="1">
-      <c r="A28" t="s" s="65">
-        <v>149</v>
-      </c>
-      <c r="B28" t="s" s="65">
-        <v>299</v>
-      </c>
-      <c r="C28" t="s" s="65">
-        <v>303</v>
-      </c>
-      <c r="D28" t="s" s="65">
-        <v>355</v>
-      </c>
-      <c r="E28" s="66">
-        <v>3</v>
-      </c>
-      <c r="F28" t="s" s="65">
-        <v>356</v>
-      </c>
-      <c r="G28" t="s" s="65">
-        <v>357</v>
-      </c>
-      <c r="H28" s="30"/>
-      <c r="I28" s="30"/>
-    </row>
-    <row r="29" ht="31.5" customHeight="1">
-      <c r="A29" t="s" s="65">
-        <v>231</v>
-      </c>
-      <c r="B29" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C29" t="s" s="65">
-        <v>317</v>
-      </c>
-      <c r="D29" t="s" s="65">
-        <v>358</v>
-      </c>
-      <c r="E29" s="66">
-        <v>3</v>
-      </c>
-      <c r="F29" t="s" s="65">
-        <v>359</v>
-      </c>
-      <c r="G29" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H29" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I29" s="30"/>
-    </row>
-    <row r="30" ht="31.5" customHeight="1">
-      <c r="A30" t="s" s="65">
-        <v>231</v>
-      </c>
-      <c r="B30" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C30" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D30" t="s" s="65">
-        <v>360</v>
-      </c>
-      <c r="E30" s="66">
-        <v>3</v>
-      </c>
-      <c r="F30" t="s" s="65">
-        <v>361</v>
-      </c>
-      <c r="G30" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H30" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I30" s="30"/>
-    </row>
-    <row r="31" ht="31.5" customHeight="1">
-      <c r="A31" t="s" s="65">
-        <v>231</v>
-      </c>
-      <c r="B31" t="s" s="65">
-        <v>299</v>
-      </c>
-      <c r="C31" t="s" s="65">
-        <v>73</v>
-      </c>
-      <c r="D31" t="s" s="65">
-        <v>362</v>
-      </c>
-      <c r="E31" s="66">
-        <v>2</v>
-      </c>
-      <c r="F31" t="s" s="65">
-        <v>363</v>
-      </c>
-      <c r="G31" t="s" s="65">
-        <v>364</v>
-      </c>
-      <c r="H31" s="30"/>
-      <c r="I31" s="30"/>
-    </row>
-    <row r="32" ht="31.5" customHeight="1">
-      <c r="A32" t="s" s="65">
-        <v>231</v>
-      </c>
-      <c r="B32" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C32" t="s" s="65">
-        <v>336</v>
-      </c>
-      <c r="D32" t="s" s="65">
-        <v>365</v>
-      </c>
-      <c r="E32" s="66">
-        <v>1</v>
-      </c>
-      <c r="F32" t="s" s="65">
-        <v>366</v>
-      </c>
-      <c r="G32" t="s" s="65">
-        <v>316</v>
-      </c>
-      <c r="H32" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I32" s="30"/>
-    </row>
-    <row r="33" ht="31.5" customHeight="1">
-      <c r="A33" t="s" s="65">
-        <v>239</v>
-      </c>
-      <c r="B33" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C33" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D33" t="s" s="65">
-        <v>367</v>
-      </c>
-      <c r="E33" s="66">
-        <v>3</v>
-      </c>
-      <c r="F33" t="s" s="65">
-        <v>368</v>
-      </c>
-      <c r="G33" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H33" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I33" s="30"/>
-    </row>
-    <row r="34" ht="31.5" customHeight="1">
-      <c r="A34" t="s" s="65">
-        <v>239</v>
-      </c>
-      <c r="B34" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C34" t="s" s="65">
-        <v>317</v>
-      </c>
-      <c r="D34" t="s" s="65">
-        <v>369</v>
-      </c>
-      <c r="E34" s="66">
-        <v>2</v>
-      </c>
-      <c r="F34" t="s" s="65">
-        <v>370</v>
-      </c>
-      <c r="G34" t="s" s="65">
-        <v>316</v>
-      </c>
-      <c r="H34" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I34" s="30"/>
-    </row>
-    <row r="35" ht="31.5" customHeight="1">
-      <c r="A35" t="s" s="67">
-        <v>239</v>
-      </c>
-      <c r="B35" t="s" s="67">
-        <v>299</v>
-      </c>
-      <c r="C35" t="s" s="67">
-        <v>291</v>
-      </c>
-      <c r="D35" t="s" s="67">
-        <v>371</v>
-      </c>
-      <c r="E35" s="68">
-        <v>3</v>
-      </c>
-      <c r="F35" t="s" s="67">
-        <v>372</v>
-      </c>
-      <c r="G35" t="s" s="67">
-        <v>373</v>
-      </c>
-      <c r="H35" s="69"/>
-      <c r="I35" s="30"/>
-    </row>
-    <row r="36" ht="31.5" customHeight="1">
-      <c r="A36" t="s" s="70">
-        <v>239</v>
-      </c>
-      <c r="B36" t="s" s="71">
-        <v>70</v>
-      </c>
-      <c r="C36" t="s" s="71">
-        <v>374</v>
-      </c>
-      <c r="D36" t="s" s="71">
-        <v>375</v>
-      </c>
-      <c r="E36" s="72">
-        <v>1</v>
-      </c>
-      <c r="F36" t="s" s="71">
-        <v>376</v>
-      </c>
-      <c r="G36" t="s" s="71">
-        <v>377</v>
-      </c>
-      <c r="H36" t="s" s="71">
-        <v>378</v>
-      </c>
-      <c r="I36" s="54"/>
-    </row>
-    <row r="37" ht="31.5" customHeight="1">
-      <c r="A37" t="s" s="63">
-        <v>247</v>
-      </c>
-      <c r="B37" t="s" s="63">
-        <v>70</v>
-      </c>
-      <c r="C37" t="s" s="63">
-        <v>73</v>
-      </c>
-      <c r="D37" t="s" s="63">
-        <v>379</v>
-      </c>
-      <c r="E37" s="64">
-        <v>3</v>
-      </c>
-      <c r="F37" t="s" s="63">
-        <v>380</v>
-      </c>
-      <c r="G37" t="s" s="63">
-        <v>322</v>
-      </c>
-      <c r="H37" t="s" s="63">
-        <v>295</v>
-      </c>
-      <c r="I37" s="30"/>
-    </row>
-    <row r="38" ht="31.5" customHeight="1">
-      <c r="A38" t="s" s="65">
-        <v>247</v>
-      </c>
-      <c r="B38" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C38" t="s" s="65">
-        <v>303</v>
-      </c>
-      <c r="D38" t="s" s="65">
-        <v>381</v>
-      </c>
-      <c r="E38" s="66">
-        <v>3</v>
-      </c>
-      <c r="F38" t="s" s="65">
-        <v>382</v>
-      </c>
-      <c r="G38" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H38" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I38" s="30"/>
-    </row>
-    <row r="39" ht="31.5" customHeight="1">
-      <c r="A39" t="s" s="65">
-        <v>247</v>
-      </c>
-      <c r="B39" t="s" s="65">
-        <v>299</v>
-      </c>
-      <c r="C39" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D39" t="s" s="65">
-        <v>383</v>
-      </c>
-      <c r="E39" s="66">
-        <v>3</v>
-      </c>
-      <c r="F39" t="s" s="65">
+      <c r="F59" t="s" s="70">
         <v>384</v>
       </c>
-      <c r="G39" t="s" s="65">
+      <c r="G59" t="s" s="70">
         <v>385</v>
       </c>
-      <c r="H39" s="30"/>
-      <c r="I39" s="30"/>
-    </row>
-    <row r="40" ht="31.5" customHeight="1">
-      <c r="A40" t="s" s="65">
-        <v>247</v>
-      </c>
-      <c r="B40" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C40" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D40" t="s" s="65">
-        <v>386</v>
-      </c>
-      <c r="E40" s="66">
-        <v>2</v>
-      </c>
-      <c r="F40" t="s" s="65">
-        <v>387</v>
-      </c>
-      <c r="G40" t="s" s="65">
-        <v>316</v>
-      </c>
-      <c r="H40" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I40" s="30"/>
-    </row>
-    <row r="41" ht="31.5" customHeight="1">
-      <c r="A41" t="s" s="65">
-        <v>255</v>
-      </c>
-      <c r="B41" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C41" t="s" s="65">
-        <v>73</v>
-      </c>
-      <c r="D41" t="s" s="65">
-        <v>388</v>
-      </c>
-      <c r="E41" s="66">
-        <v>3</v>
-      </c>
-      <c r="F41" t="s" s="65">
-        <v>389</v>
-      </c>
-      <c r="G41" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H41" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I41" s="30"/>
-    </row>
-    <row r="42" ht="31.5" customHeight="1">
-      <c r="A42" t="s" s="65">
-        <v>255</v>
-      </c>
-      <c r="B42" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C42" t="s" s="65">
-        <v>303</v>
-      </c>
-      <c r="D42" t="s" s="65">
-        <v>390</v>
-      </c>
-      <c r="E42" s="66">
-        <v>3</v>
-      </c>
-      <c r="F42" t="s" s="65">
-        <v>391</v>
-      </c>
-      <c r="G42" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H42" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I42" s="30"/>
-    </row>
-    <row r="43" ht="31.5" customHeight="1">
-      <c r="A43" t="s" s="65">
-        <v>255</v>
-      </c>
-      <c r="B43" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C43" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D43" t="s" s="65">
-        <v>392</v>
-      </c>
-      <c r="E43" s="66">
-        <v>2</v>
-      </c>
-      <c r="F43" t="s" s="65">
-        <v>393</v>
-      </c>
-      <c r="G43" t="s" s="65">
-        <v>316</v>
-      </c>
-      <c r="H43" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I43" s="30"/>
-    </row>
-    <row r="44" ht="31.5" customHeight="1">
-      <c r="A44" t="s" s="65">
-        <v>255</v>
-      </c>
-      <c r="B44" t="s" s="65">
-        <v>299</v>
-      </c>
-      <c r="C44" t="s" s="65">
-        <v>303</v>
-      </c>
-      <c r="D44" t="s" s="65">
-        <v>394</v>
-      </c>
-      <c r="E44" s="66">
-        <v>2</v>
-      </c>
-      <c r="F44" t="s" s="65">
-        <v>395</v>
-      </c>
-      <c r="G44" t="s" s="65">
-        <v>373</v>
-      </c>
-      <c r="H44" s="30"/>
-      <c r="I44" s="30"/>
-    </row>
-    <row r="45" ht="31.5" customHeight="1">
-      <c r="A45" t="s" s="65">
-        <v>263</v>
-      </c>
-      <c r="B45" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C45" t="s" s="65">
-        <v>317</v>
-      </c>
-      <c r="D45" t="s" s="65">
-        <v>396</v>
-      </c>
-      <c r="E45" s="66">
-        <v>3</v>
-      </c>
-      <c r="F45" t="s" s="65">
-        <v>397</v>
-      </c>
-      <c r="G45" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H45" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I45" s="30"/>
-    </row>
-    <row r="46" ht="31.5" customHeight="1">
-      <c r="A46" t="s" s="65">
-        <v>263</v>
-      </c>
-      <c r="B46" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C46" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D46" t="s" s="65">
-        <v>398</v>
-      </c>
-      <c r="E46" s="66">
-        <v>3</v>
-      </c>
-      <c r="F46" t="s" s="65">
-        <v>399</v>
-      </c>
-      <c r="G46" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H46" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I46" s="30"/>
-    </row>
-    <row r="47" ht="31.5" customHeight="1">
-      <c r="A47" t="s" s="65">
-        <v>263</v>
-      </c>
-      <c r="B47" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C47" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D47" t="s" s="65">
-        <v>400</v>
-      </c>
-      <c r="E47" s="66">
-        <v>3</v>
-      </c>
-      <c r="F47" t="s" s="65">
-        <v>401</v>
-      </c>
-      <c r="G47" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H47" t="s" s="65">
-        <v>295</v>
-      </c>
-      <c r="I47" s="30"/>
-    </row>
-    <row r="48" ht="31.5" customHeight="1">
-      <c r="A48" t="s" s="65">
-        <v>263</v>
-      </c>
-      <c r="B48" t="s" s="65">
-        <v>299</v>
-      </c>
-      <c r="C48" t="s" s="65">
-        <v>303</v>
-      </c>
-      <c r="D48" t="s" s="65">
-        <v>402</v>
-      </c>
-      <c r="E48" s="66">
-        <v>2</v>
-      </c>
-      <c r="F48" t="s" s="65">
-        <v>403</v>
-      </c>
-      <c r="G48" t="s" s="65">
-        <v>404</v>
-      </c>
-      <c r="H48" s="30"/>
-      <c r="I48" s="30"/>
-    </row>
-    <row r="49" ht="31.5" customHeight="1">
-      <c r="A49" t="s" s="73">
-        <v>271</v>
-      </c>
-      <c r="B49" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C49" t="s" s="65">
-        <v>317</v>
-      </c>
-      <c r="D49" t="s" s="65">
-        <v>405</v>
-      </c>
-      <c r="E49" s="66">
-        <v>3</v>
-      </c>
-      <c r="F49" t="s" s="65">
-        <v>406</v>
-      </c>
-      <c r="G49" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H49" s="74"/>
-      <c r="I49" s="29"/>
-    </row>
-    <row r="50" ht="31.5" customHeight="1">
-      <c r="A50" t="s" s="73">
-        <v>271</v>
-      </c>
-      <c r="B50" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C50" t="s" s="65">
-        <v>303</v>
-      </c>
-      <c r="D50" t="s" s="65">
-        <v>407</v>
-      </c>
-      <c r="E50" s="66">
-        <v>3</v>
-      </c>
-      <c r="F50" t="s" s="65">
-        <v>408</v>
-      </c>
-      <c r="G50" t="s" s="65">
-        <v>322</v>
-      </c>
-      <c r="H50" s="74"/>
-      <c r="I50" s="29"/>
-    </row>
-    <row r="51" ht="31.5" customHeight="1">
-      <c r="A51" t="s" s="73">
-        <v>271</v>
-      </c>
-      <c r="B51" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C51" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D51" t="s" s="65">
-        <v>409</v>
-      </c>
-      <c r="E51" s="66">
-        <v>2</v>
-      </c>
-      <c r="F51" t="s" s="65">
-        <v>410</v>
-      </c>
-      <c r="G51" t="s" s="65">
-        <v>316</v>
-      </c>
-      <c r="H51" s="74"/>
-      <c r="I51" s="29"/>
-    </row>
-    <row r="52" ht="31.5" customHeight="1">
-      <c r="A52" t="s" s="73">
-        <v>271</v>
-      </c>
-      <c r="B52" t="s" s="65">
-        <v>299</v>
-      </c>
-      <c r="C52" t="s" s="65">
-        <v>73</v>
-      </c>
-      <c r="D52" t="s" s="65">
-        <v>411</v>
-      </c>
-      <c r="E52" s="66">
-        <v>3</v>
-      </c>
-      <c r="F52" t="s" s="65">
-        <v>412</v>
-      </c>
-      <c r="G52" t="s" s="65">
-        <v>345</v>
-      </c>
-      <c r="H52" s="74"/>
-      <c r="I52" s="29"/>
-    </row>
-    <row r="53" ht="31.5" customHeight="1">
-      <c r="A53" t="s" s="73">
-        <v>271</v>
-      </c>
-      <c r="B53" t="s" s="65">
-        <v>299</v>
-      </c>
-      <c r="C53" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D53" t="s" s="65">
-        <v>413</v>
-      </c>
-      <c r="E53" s="66">
-        <v>2</v>
-      </c>
-      <c r="F53" t="s" s="65">
-        <v>414</v>
-      </c>
-      <c r="G53" t="s" s="65">
-        <v>404</v>
-      </c>
-      <c r="H53" s="74"/>
-      <c r="I53" s="29"/>
-    </row>
-    <row r="54" ht="31.5" customHeight="1">
-      <c r="A54" t="s" s="73">
-        <v>280</v>
-      </c>
-      <c r="B54" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C54" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D54" t="s" s="65">
-        <v>415</v>
-      </c>
-      <c r="E54" s="66">
-        <v>3</v>
-      </c>
-      <c r="F54" t="s" s="65">
-        <v>416</v>
-      </c>
-      <c r="G54" t="s" s="65">
-        <v>417</v>
-      </c>
-      <c r="H54" t="s" s="75">
-        <v>418</v>
-      </c>
-      <c r="I54" s="29"/>
-    </row>
-    <row r="55" ht="31.5" customHeight="1">
-      <c r="A55" t="s" s="73">
-        <v>280</v>
-      </c>
-      <c r="B55" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C55" t="s" s="65">
-        <v>317</v>
-      </c>
-      <c r="D55" t="s" s="65">
-        <v>419</v>
-      </c>
-      <c r="E55" s="66">
-        <v>2</v>
-      </c>
-      <c r="F55" t="s" s="65">
-        <v>420</v>
-      </c>
-      <c r="G55" t="s" s="65">
-        <v>316</v>
-      </c>
-      <c r="H55" t="s" s="75">
-        <v>421</v>
-      </c>
-      <c r="I55" s="29"/>
-    </row>
-    <row r="56" ht="31.5" customHeight="1">
-      <c r="A56" t="s" s="73">
-        <v>280</v>
-      </c>
-      <c r="B56" t="s" s="65">
-        <v>70</v>
-      </c>
-      <c r="C56" t="s" s="65">
-        <v>422</v>
-      </c>
-      <c r="D56" t="s" s="65">
-        <v>423</v>
-      </c>
-      <c r="E56" s="66">
-        <v>2</v>
-      </c>
-      <c r="F56" t="s" s="65">
-        <v>424</v>
-      </c>
-      <c r="G56" t="s" s="65">
-        <v>316</v>
-      </c>
-      <c r="H56" s="74"/>
-      <c r="I56" s="29"/>
-    </row>
-    <row r="57" ht="31.5" customHeight="1">
-      <c r="A57" t="s" s="73">
-        <v>280</v>
-      </c>
-      <c r="B57" t="s" s="65">
-        <v>299</v>
-      </c>
-      <c r="C57" t="s" s="65">
-        <v>291</v>
-      </c>
-      <c r="D57" t="s" s="65">
-        <v>425</v>
-      </c>
-      <c r="E57" s="66">
-        <v>3</v>
-      </c>
-      <c r="F57" t="s" s="65">
-        <v>384</v>
-      </c>
-      <c r="G57" t="s" s="65">
-        <v>385</v>
-      </c>
-      <c r="H57" t="s" s="75">
-        <v>426</v>
-      </c>
-      <c r="I57" s="29"/>
-    </row>
-    <row r="58" ht="19" customHeight="1">
-      <c r="A58" t="s" s="73">
-        <v>280</v>
-      </c>
-      <c r="B58" t="s" s="65">
-        <v>299</v>
-      </c>
-      <c r="C58" t="s" s="65">
-        <v>422</v>
-      </c>
-      <c r="D58" t="s" s="65">
-        <v>427</v>
-      </c>
-      <c r="E58" s="66">
-        <v>2</v>
-      </c>
-      <c r="F58" t="s" s="65">
-        <v>384</v>
-      </c>
-      <c r="G58" t="s" s="65">
-        <v>385</v>
-      </c>
-      <c r="H58" s="74"/>
-      <c r="I58" s="29"/>
+      <c r="H59" s="80"/>
+      <c r="I59" s="29"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -7620,14 +7612,14 @@
   <dimension ref="A1:G21"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="14.1719" style="76" customWidth="1"/>
-    <col min="2" max="2" width="16.6719" style="76" customWidth="1"/>
-    <col min="3" max="3" width="42.1719" style="76" customWidth="1"/>
-    <col min="4" max="4" width="32" style="76" customWidth="1"/>
-    <col min="5" max="5" width="33.3516" style="76" customWidth="1"/>
-    <col min="6" max="6" width="32.8516" style="76" customWidth="1"/>
-    <col min="7" max="7" width="40" style="76" customWidth="1"/>
-    <col min="8" max="16384" width="8.85156" style="76" customWidth="1"/>
+    <col min="1" max="1" width="14.1719" style="82" customWidth="1"/>
+    <col min="2" max="2" width="16.6719" style="82" customWidth="1"/>
+    <col min="3" max="3" width="42.1719" style="82" customWidth="1"/>
+    <col min="4" max="4" width="32" style="82" customWidth="1"/>
+    <col min="5" max="5" width="33.3516" style="82" customWidth="1"/>
+    <col min="6" max="6" width="32.8516" style="82" customWidth="1"/>
+    <col min="7" max="7" width="40" style="82" customWidth="1"/>
+    <col min="8" max="16384" width="8.85156" style="82" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="47" customHeight="1">
@@ -7691,10 +7683,10 @@
       <c r="B5" t="s" s="32">
         <v>97</v>
       </c>
-      <c r="C5" t="s" s="77">
+      <c r="C5" t="s" s="55">
         <v>430</v>
       </c>
-      <c r="D5" t="s" s="77">
+      <c r="D5" t="s" s="55">
         <v>431</v>
       </c>
       <c r="E5" t="s" s="32">
@@ -7707,17 +7699,17 @@
         <v>434</v>
       </c>
     </row>
-    <row r="6" ht="35" customHeight="1">
+    <row r="6" ht="51" customHeight="1">
       <c r="A6" t="s" s="34">
         <v>33</v>
       </c>
       <c r="B6" t="s" s="35">
         <v>125</v>
       </c>
-      <c r="C6" t="s" s="35">
+      <c r="C6" t="s" s="57">
         <v>435</v>
       </c>
-      <c r="D6" t="s" s="35">
+      <c r="D6" t="s" s="57">
         <v>436</v>
       </c>
       <c r="E6" t="s" s="35">
@@ -7737,10 +7729,10 @@
       <c r="B7" t="s" s="33">
         <v>149</v>
       </c>
-      <c r="C7" t="s" s="31">
+      <c r="C7" t="s" s="83">
         <v>440</v>
       </c>
-      <c r="D7" t="s" s="33">
+      <c r="D7" t="s" s="84">
         <v>441</v>
       </c>
       <c r="E7" t="s" s="31">
@@ -7749,7 +7741,7 @@
       <c r="F7" t="s" s="33">
         <v>433</v>
       </c>
-      <c r="G7" t="s" s="78">
+      <c r="G7" t="s" s="85">
         <v>443</v>
       </c>
     </row>
@@ -7795,7 +7787,7 @@
       <c r="F9" t="s" s="33">
         <v>447</v>
       </c>
-      <c r="G9" t="s" s="78">
+      <c r="G9" t="s" s="85">
         <v>452</v>
       </c>
     </row>
@@ -7841,7 +7833,7 @@
       <c r="F11" t="s" s="33">
         <v>461</v>
       </c>
-      <c r="G11" t="s" s="78">
+      <c r="G11" t="s" s="85">
         <v>462</v>
       </c>
     </row>
@@ -7887,7 +7879,7 @@
       <c r="F13" t="s" s="33">
         <v>471</v>
       </c>
-      <c r="G13" t="s" s="78">
+      <c r="G13" t="s" s="85">
         <v>472</v>
       </c>
     </row>
@@ -7933,7 +7925,7 @@
       <c r="F15" t="s" s="33">
         <v>447</v>
       </c>
-      <c r="G15" t="s" s="78">
+      <c r="G15" t="s" s="85">
         <v>480</v>
       </c>
     </row>
@@ -7979,7 +7971,7 @@
       <c r="F17" t="s" s="33">
         <v>489</v>
       </c>
-      <c r="G17" t="s" s="78">
+      <c r="G17" t="s" s="85">
         <v>490</v>
       </c>
     </row>
@@ -8025,7 +8017,7 @@
       <c r="F19" t="s" s="33">
         <v>447</v>
       </c>
-      <c r="G19" t="s" s="78">
+      <c r="G19" t="s" s="85">
         <v>499</v>
       </c>
     </row>
@@ -8071,7 +8063,7 @@
       <c r="F21" t="s" s="33">
         <v>507</v>
       </c>
-      <c r="G21" t="s" s="78">
+      <c r="G21" t="s" s="85">
         <v>508</v>
       </c>
     </row>
@@ -8089,16 +8081,16 @@
   <dimension ref="A1:I17"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="10" style="79" customWidth="1"/>
-    <col min="2" max="2" width="13.5" style="79" customWidth="1"/>
-    <col min="3" max="3" width="11.6719" style="79" customWidth="1"/>
-    <col min="4" max="4" width="39.3516" style="79" customWidth="1"/>
-    <col min="5" max="5" width="33.3516" style="79" customWidth="1"/>
-    <col min="6" max="6" width="15.5" style="79" customWidth="1"/>
-    <col min="7" max="7" width="40" style="79" customWidth="1"/>
-    <col min="8" max="8" width="19.1719" style="79" customWidth="1"/>
-    <col min="9" max="9" width="8.85156" style="79" customWidth="1"/>
-    <col min="10" max="16384" width="8.85156" style="79" customWidth="1"/>
+    <col min="1" max="1" width="10" style="86" customWidth="1"/>
+    <col min="2" max="2" width="13.5" style="86" customWidth="1"/>
+    <col min="3" max="3" width="11.6719" style="86" customWidth="1"/>
+    <col min="4" max="4" width="39.3516" style="86" customWidth="1"/>
+    <col min="5" max="5" width="33.3516" style="86" customWidth="1"/>
+    <col min="6" max="6" width="15.5" style="86" customWidth="1"/>
+    <col min="7" max="7" width="40" style="86" customWidth="1"/>
+    <col min="8" max="8" width="19.1719" style="86" customWidth="1"/>
+    <col min="9" max="9" width="8.85156" style="86" customWidth="1"/>
+    <col min="10" max="16384" width="8.85156" style="86" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="72.5" customHeight="1">
@@ -8169,7 +8161,7 @@
       <c r="A5" t="s" s="31">
         <v>121</v>
       </c>
-      <c r="B5" s="80"/>
+      <c r="B5" s="87"/>
       <c r="C5" t="s" s="32">
         <v>129</v>
       </c>
@@ -8243,249 +8235,249 @@
       <c r="I7" s="29"/>
     </row>
     <row r="8" ht="53.4" customHeight="1">
-      <c r="A8" t="s" s="81">
+      <c r="A8" t="s" s="88">
         <v>121</v>
       </c>
       <c r="B8" s="40"/>
-      <c r="C8" t="s" s="82">
+      <c r="C8" t="s" s="89">
         <v>524</v>
       </c>
-      <c r="D8" t="s" s="82">
+      <c r="D8" t="s" s="89">
         <v>525</v>
       </c>
-      <c r="E8" t="s" s="82">
+      <c r="E8" t="s" s="89">
         <v>526</v>
       </c>
-      <c r="F8" t="s" s="82">
+      <c r="F8" t="s" s="89">
         <v>517</v>
       </c>
-      <c r="G8" t="s" s="82">
+      <c r="G8" t="s" s="89">
         <v>527</v>
       </c>
-      <c r="H8" t="s" s="83">
+      <c r="H8" t="s" s="90">
         <v>528</v>
       </c>
       <c r="I8" s="29"/>
     </row>
     <row r="9" ht="35" customHeight="1">
-      <c r="A9" t="s" s="73">
+      <c r="A9" t="s" s="79">
         <v>121</v>
       </c>
       <c r="B9" s="30"/>
-      <c r="C9" t="s" s="65">
+      <c r="C9" t="s" s="70">
         <v>524</v>
       </c>
-      <c r="D9" t="s" s="65">
+      <c r="D9" t="s" s="70">
         <v>529</v>
       </c>
-      <c r="E9" t="s" s="65">
+      <c r="E9" t="s" s="70">
         <v>512</v>
       </c>
-      <c r="F9" t="s" s="65">
+      <c r="F9" t="s" s="70">
         <v>517</v>
       </c>
-      <c r="G9" t="s" s="65">
+      <c r="G9" t="s" s="70">
         <v>530</v>
       </c>
-      <c r="H9" s="74"/>
+      <c r="H9" s="80"/>
       <c r="I9" s="29"/>
     </row>
     <row r="10" ht="51" customHeight="1">
-      <c r="A10" t="s" s="73">
+      <c r="A10" t="s" s="79">
         <v>121</v>
       </c>
       <c r="B10" s="30"/>
-      <c r="C10" t="s" s="65">
+      <c r="C10" t="s" s="70">
         <v>531</v>
       </c>
-      <c r="D10" t="s" s="65">
+      <c r="D10" t="s" s="70">
         <v>532</v>
       </c>
-      <c r="E10" t="s" s="65">
+      <c r="E10" t="s" s="70">
         <v>533</v>
       </c>
-      <c r="F10" t="s" s="65">
+      <c r="F10" t="s" s="70">
         <v>141</v>
       </c>
-      <c r="G10" t="s" s="65">
+      <c r="G10" t="s" s="70">
         <v>534</v>
       </c>
-      <c r="H10" t="s" s="75">
+      <c r="H10" t="s" s="81">
         <v>535</v>
       </c>
       <c r="I10" s="29"/>
     </row>
     <row r="11" ht="35" customHeight="1">
-      <c r="A11" t="s" s="73">
+      <c r="A11" t="s" s="79">
         <v>121</v>
       </c>
       <c r="B11" s="30"/>
-      <c r="C11" t="s" s="65">
+      <c r="C11" t="s" s="70">
         <v>129</v>
       </c>
-      <c r="D11" t="s" s="65">
+      <c r="D11" t="s" s="70">
         <v>536</v>
       </c>
-      <c r="E11" t="s" s="65">
+      <c r="E11" t="s" s="70">
         <v>537</v>
       </c>
-      <c r="F11" t="s" s="65">
+      <c r="F11" t="s" s="70">
         <v>141</v>
       </c>
-      <c r="G11" t="s" s="65">
+      <c r="G11" t="s" s="70">
         <v>538</v>
       </c>
-      <c r="H11" s="74"/>
+      <c r="H11" s="80"/>
       <c r="I11" s="29"/>
     </row>
     <row r="12" ht="35" customHeight="1">
-      <c r="A12" t="s" s="73">
+      <c r="A12" t="s" s="79">
         <v>121</v>
       </c>
       <c r="B12" s="30"/>
-      <c r="C12" t="s" s="65">
+      <c r="C12" t="s" s="70">
         <v>514</v>
       </c>
-      <c r="D12" t="s" s="65">
+      <c r="D12" t="s" s="70">
         <v>539</v>
       </c>
-      <c r="E12" t="s" s="65">
+      <c r="E12" t="s" s="70">
         <v>540</v>
       </c>
-      <c r="F12" t="s" s="65">
+      <c r="F12" t="s" s="70">
         <v>141</v>
       </c>
-      <c r="G12" t="s" s="65">
+      <c r="G12" t="s" s="70">
         <v>541</v>
       </c>
-      <c r="H12" s="74"/>
+      <c r="H12" s="80"/>
       <c r="I12" s="29"/>
     </row>
     <row r="13" ht="51" customHeight="1">
-      <c r="A13" t="s" s="73">
+      <c r="A13" t="s" s="79">
         <v>121</v>
       </c>
       <c r="B13" s="30"/>
-      <c r="C13" t="s" s="65">
+      <c r="C13" t="s" s="70">
         <v>542</v>
       </c>
-      <c r="D13" t="s" s="65">
+      <c r="D13" t="s" s="70">
         <v>543</v>
       </c>
-      <c r="E13" t="s" s="65">
+      <c r="E13" t="s" s="70">
         <v>544</v>
       </c>
-      <c r="F13" t="s" s="65">
+      <c r="F13" t="s" s="70">
         <v>141</v>
       </c>
-      <c r="G13" t="s" s="65">
+      <c r="G13" t="s" s="70">
         <v>545</v>
       </c>
-      <c r="H13" t="s" s="75">
+      <c r="H13" t="s" s="81">
         <v>546</v>
       </c>
       <c r="I13" s="29"/>
     </row>
     <row r="14" ht="51" customHeight="1">
-      <c r="A14" t="s" s="73">
+      <c r="A14" t="s" s="79">
         <v>519</v>
       </c>
-      <c r="B14" t="s" s="65">
+      <c r="B14" t="s" s="70">
         <v>239</v>
       </c>
-      <c r="C14" t="s" s="65">
+      <c r="C14" t="s" s="70">
         <v>129</v>
       </c>
-      <c r="D14" t="s" s="65">
+      <c r="D14" t="s" s="70">
         <v>547</v>
       </c>
-      <c r="E14" t="s" s="65">
+      <c r="E14" t="s" s="70">
         <v>548</v>
       </c>
-      <c r="F14" t="s" s="65">
+      <c r="F14" t="s" s="70">
         <v>517</v>
       </c>
-      <c r="G14" t="s" s="65">
+      <c r="G14" t="s" s="70">
         <v>549</v>
       </c>
-      <c r="H14" t="s" s="75">
+      <c r="H14" t="s" s="81">
         <v>550</v>
       </c>
       <c r="I14" s="29"/>
     </row>
     <row r="15" ht="35" customHeight="1">
-      <c r="A15" t="s" s="73">
+      <c r="A15" t="s" s="79">
         <v>519</v>
       </c>
-      <c r="B15" t="s" s="65">
+      <c r="B15" t="s" s="70">
         <v>280</v>
       </c>
-      <c r="C15" t="s" s="65">
+      <c r="C15" t="s" s="70">
         <v>129</v>
       </c>
-      <c r="D15" t="s" s="65">
+      <c r="D15" t="s" s="70">
         <v>547</v>
       </c>
-      <c r="E15" t="s" s="65">
+      <c r="E15" t="s" s="70">
         <v>548</v>
       </c>
-      <c r="F15" t="s" s="65">
+      <c r="F15" t="s" s="70">
         <v>517</v>
       </c>
-      <c r="G15" t="s" s="65">
+      <c r="G15" t="s" s="70">
         <v>551</v>
       </c>
-      <c r="H15" s="74"/>
+      <c r="H15" s="80"/>
       <c r="I15" s="29"/>
     </row>
     <row r="16" ht="37.4" customHeight="1">
-      <c r="A16" t="s" s="73">
+      <c r="A16" t="s" s="79">
         <v>519</v>
       </c>
-      <c r="B16" t="s" s="65">
+      <c r="B16" t="s" s="70">
         <v>247</v>
       </c>
-      <c r="C16" t="s" s="65">
+      <c r="C16" t="s" s="70">
         <v>129</v>
       </c>
-      <c r="D16" t="s" s="65">
+      <c r="D16" t="s" s="70">
         <v>552</v>
       </c>
-      <c r="E16" t="s" s="65">
+      <c r="E16" t="s" s="70">
         <v>553</v>
       </c>
-      <c r="F16" t="s" s="65">
+      <c r="F16" t="s" s="70">
         <v>141</v>
       </c>
-      <c r="G16" t="s" s="65">
+      <c r="G16" t="s" s="70">
         <v>554</v>
       </c>
-      <c r="H16" s="74"/>
+      <c r="H16" s="80"/>
       <c r="I16" s="29"/>
     </row>
     <row r="17" ht="37.4" customHeight="1">
-      <c r="A17" t="s" s="73">
+      <c r="A17" t="s" s="79">
         <v>519</v>
       </c>
-      <c r="B17" t="s" s="65">
+      <c r="B17" t="s" s="70">
         <v>255</v>
       </c>
-      <c r="C17" t="s" s="65">
+      <c r="C17" t="s" s="70">
         <v>129</v>
       </c>
-      <c r="D17" t="s" s="65">
+      <c r="D17" t="s" s="70">
         <v>555</v>
       </c>
-      <c r="E17" t="s" s="65">
+      <c r="E17" t="s" s="70">
         <v>556</v>
       </c>
-      <c r="F17" t="s" s="65">
+      <c r="F17" t="s" s="70">
         <v>141</v>
       </c>
-      <c r="G17" t="s" s="65">
+      <c r="G17" t="s" s="70">
         <v>557</v>
       </c>
-      <c r="H17" s="74"/>
+      <c r="H17" s="80"/>
       <c r="I17" s="29"/>
     </row>
   </sheetData>
@@ -8499,18 +8491,19 @@
 
 <file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <dimension ref="A1:I39"/>
+  <dimension ref="A1:I38"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="14.1719" style="84" customWidth="1"/>
-    <col min="2" max="2" width="23.3516" style="84" customWidth="1"/>
-    <col min="3" max="4" width="26.5" style="84" customWidth="1"/>
-    <col min="5" max="5" width="6.67188" style="84" customWidth="1"/>
-    <col min="6" max="6" width="46.6719" style="84" customWidth="1"/>
-    <col min="7" max="7" width="17.3516" style="84" customWidth="1"/>
-    <col min="8" max="8" width="10.6719" style="84" customWidth="1"/>
-    <col min="9" max="9" width="8.85156" style="84" customWidth="1"/>
-    <col min="10" max="16384" width="8.85156" style="84" customWidth="1"/>
+    <col min="1" max="1" width="14.1719" style="91" customWidth="1"/>
+    <col min="2" max="2" width="23.3516" style="91" customWidth="1"/>
+    <col min="3" max="3" width="26.5" style="91" customWidth="1"/>
+    <col min="4" max="4" width="35.6719" style="91" customWidth="1"/>
+    <col min="5" max="5" width="6.67188" style="91" customWidth="1"/>
+    <col min="6" max="6" width="46.6719" style="91" customWidth="1"/>
+    <col min="7" max="7" width="17.3516" style="91" customWidth="1"/>
+    <col min="8" max="8" width="10.6719" style="91" customWidth="1"/>
+    <col min="9" max="9" width="8.85156" style="91" customWidth="1"/>
+    <col min="10" max="16384" width="8.85156" style="91" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="47" customHeight="1">
@@ -8590,7 +8583,7 @@
       <c r="D5" t="s" s="32">
         <v>562</v>
       </c>
-      <c r="E5" s="55">
+      <c r="E5" s="56">
         <v>1</v>
       </c>
       <c r="F5" t="s" s="32">
@@ -8605,910 +8598,885 @@
       <c r="I5" s="29"/>
     </row>
     <row r="6" ht="35" customHeight="1">
-      <c r="A6" t="s" s="85">
+      <c r="A6" t="s" s="92">
         <v>33</v>
       </c>
-      <c r="B6" t="s" s="86">
+      <c r="B6" t="s" s="93">
         <v>565</v>
       </c>
-      <c r="C6" t="s" s="86">
+      <c r="C6" t="s" s="93">
         <v>566</v>
       </c>
-      <c r="D6" t="s" s="86">
+      <c r="D6" t="s" s="93">
         <v>567</v>
       </c>
-      <c r="E6" s="87">
+      <c r="E6" s="94">
         <v>1</v>
       </c>
-      <c r="F6" t="s" s="86">
+      <c r="F6" t="s" s="93">
         <v>568</v>
       </c>
-      <c r="G6" t="s" s="86">
+      <c r="G6" t="s" s="93">
         <v>569</v>
       </c>
-      <c r="H6" t="s" s="88">
+      <c r="H6" t="s" s="95">
         <v>295</v>
       </c>
       <c r="I6" s="29"/>
     </row>
     <row r="7" ht="37.4" customHeight="1">
-      <c r="A7" t="s" s="82">
+      <c r="A7" t="s" s="89">
         <v>33</v>
       </c>
-      <c r="B7" t="s" s="82">
+      <c r="B7" t="s" s="89">
         <v>570</v>
       </c>
-      <c r="C7" t="s" s="82">
+      <c r="C7" t="s" s="89">
         <v>571</v>
       </c>
-      <c r="D7" t="s" s="82">
+      <c r="D7" t="s" s="89">
         <v>572</v>
       </c>
-      <c r="E7" s="89">
+      <c r="E7" s="96">
         <v>2</v>
       </c>
-      <c r="F7" t="s" s="82">
+      <c r="F7" t="s" s="89">
         <v>573</v>
       </c>
-      <c r="G7" t="s" s="82">
+      <c r="G7" t="s" s="89">
         <v>574</v>
       </c>
-      <c r="H7" t="s" s="82">
+      <c r="H7" t="s" s="89">
         <v>295</v>
       </c>
       <c r="I7" s="30"/>
     </row>
     <row r="8" ht="35" customHeight="1">
-      <c r="A8" t="s" s="65">
+      <c r="A8" t="s" s="70">
         <v>125</v>
       </c>
-      <c r="B8" t="s" s="65">
+      <c r="B8" t="s" s="70">
         <v>575</v>
       </c>
-      <c r="C8" t="s" s="65">
+      <c r="C8" t="s" s="70">
         <v>576</v>
       </c>
-      <c r="D8" t="s" s="65">
+      <c r="D8" t="s" s="70">
         <v>577</v>
       </c>
-      <c r="E8" s="66">
+      <c r="E8" s="72">
         <v>1</v>
       </c>
-      <c r="F8" t="s" s="65">
+      <c r="F8" t="s" s="70">
         <v>578</v>
       </c>
-      <c r="G8" t="s" s="65">
+      <c r="G8" t="s" s="70">
         <v>579</v>
       </c>
-      <c r="H8" t="s" s="65">
+      <c r="H8" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I8" s="30"/>
     </row>
     <row r="9" ht="19" customHeight="1">
-      <c r="A9" t="s" s="65">
+      <c r="A9" t="s" s="70">
         <v>125</v>
       </c>
-      <c r="B9" t="s" s="65">
+      <c r="B9" t="s" s="70">
         <v>580</v>
       </c>
-      <c r="C9" t="s" s="65">
+      <c r="C9" t="s" s="70">
         <v>581</v>
       </c>
-      <c r="D9" t="s" s="65">
+      <c r="D9" t="s" s="70">
         <v>582</v>
       </c>
-      <c r="E9" s="66">
+      <c r="E9" s="72">
         <v>1</v>
       </c>
-      <c r="F9" t="s" s="65">
+      <c r="F9" t="s" s="70">
         <v>583</v>
       </c>
-      <c r="G9" t="s" s="65">
+      <c r="G9" t="s" s="70">
         <v>584</v>
       </c>
-      <c r="H9" t="s" s="65">
+      <c r="H9" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I9" s="30"/>
     </row>
     <row r="10" ht="35" customHeight="1">
-      <c r="A10" t="s" s="65">
+      <c r="A10" t="s" s="70">
         <v>125</v>
       </c>
-      <c r="B10" t="s" s="65">
+      <c r="B10" t="s" s="70">
         <v>585</v>
       </c>
-      <c r="C10" t="s" s="65">
+      <c r="C10" t="s" s="70">
         <v>586</v>
       </c>
-      <c r="D10" t="s" s="65">
+      <c r="D10" t="s" s="70">
         <v>587</v>
       </c>
-      <c r="E10" s="66">
+      <c r="E10" s="72">
         <v>2</v>
       </c>
-      <c r="F10" t="s" s="65">
+      <c r="F10" t="s" s="70">
         <v>588</v>
       </c>
-      <c r="G10" t="s" s="65">
+      <c r="G10" t="s" s="70">
         <v>589</v>
       </c>
-      <c r="H10" t="s" s="65">
+      <c r="H10" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I10" s="30"/>
     </row>
     <row r="11" ht="35" customHeight="1">
-      <c r="A11" t="s" s="65">
+      <c r="A11" t="s" s="70">
         <v>97</v>
       </c>
-      <c r="B11" t="s" s="65">
+      <c r="B11" t="s" s="70">
         <v>590</v>
       </c>
-      <c r="C11" t="s" s="65">
+      <c r="C11" t="s" s="70">
         <v>591</v>
       </c>
-      <c r="D11" t="s" s="65">
+      <c r="D11" t="s" s="70">
         <v>592</v>
       </c>
-      <c r="E11" s="66">
+      <c r="E11" s="72">
         <v>1</v>
       </c>
-      <c r="F11" t="s" s="65">
+      <c r="F11" t="s" s="70">
         <v>593</v>
       </c>
-      <c r="G11" t="s" s="65">
+      <c r="G11" t="s" s="70">
         <v>594</v>
       </c>
-      <c r="H11" t="s" s="65">
+      <c r="H11" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I11" s="30"/>
     </row>
     <row r="12" ht="35" customHeight="1">
-      <c r="A12" t="s" s="65">
+      <c r="A12" t="s" s="70">
         <v>97</v>
       </c>
-      <c r="B12" t="s" s="65">
+      <c r="B12" t="s" s="70">
         <v>595</v>
       </c>
-      <c r="C12" t="s" s="65">
+      <c r="C12" t="s" s="70">
         <v>596</v>
       </c>
-      <c r="D12" t="s" s="65">
+      <c r="D12" t="s" s="70">
         <v>597</v>
       </c>
-      <c r="E12" s="66">
+      <c r="E12" s="72">
         <v>1</v>
       </c>
-      <c r="F12" t="s" s="65">
+      <c r="F12" t="s" s="70">
         <v>598</v>
       </c>
-      <c r="G12" t="s" s="65">
+      <c r="G12" t="s" s="70">
         <v>599</v>
       </c>
-      <c r="H12" t="s" s="65">
+      <c r="H12" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I12" s="30"/>
     </row>
     <row r="13" ht="35" customHeight="1">
-      <c r="A13" t="s" s="65">
+      <c r="A13" t="s" s="70">
         <v>97</v>
       </c>
-      <c r="B13" t="s" s="65">
+      <c r="B13" t="s" s="70">
         <v>600</v>
       </c>
-      <c r="C13" t="s" s="65">
+      <c r="C13" t="s" s="70">
         <v>601</v>
       </c>
-      <c r="D13" t="s" s="65">
+      <c r="D13" t="s" s="70">
         <v>602</v>
       </c>
-      <c r="E13" s="66">
+      <c r="E13" s="72">
         <v>2</v>
       </c>
-      <c r="F13" t="s" s="65">
+      <c r="F13" t="s" s="70">
         <v>603</v>
       </c>
-      <c r="G13" t="s" s="65">
+      <c r="G13" t="s" s="70">
         <v>604</v>
       </c>
-      <c r="H13" t="s" s="65">
+      <c r="H13" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I13" s="30"/>
     </row>
     <row r="14" ht="19" customHeight="1">
-      <c r="A14" t="s" s="65">
+      <c r="A14" t="s" s="70">
         <v>207</v>
       </c>
-      <c r="B14" t="s" s="65">
+      <c r="B14" t="s" s="70">
         <v>605</v>
       </c>
-      <c r="C14" t="s" s="65">
+      <c r="C14" t="s" s="70">
         <v>606</v>
       </c>
-      <c r="D14" t="s" s="65">
+      <c r="D14" t="s" s="70">
         <v>607</v>
       </c>
-      <c r="E14" s="66">
+      <c r="E14" s="72">
         <v>1</v>
       </c>
-      <c r="F14" t="s" s="65">
+      <c r="F14" t="s" s="70">
         <v>608</v>
       </c>
-      <c r="G14" t="s" s="65">
+      <c r="G14" t="s" s="70">
         <v>609</v>
       </c>
-      <c r="H14" t="s" s="65">
+      <c r="H14" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I14" s="30"/>
     </row>
     <row r="15" ht="35" customHeight="1">
-      <c r="A15" t="s" s="65">
+      <c r="A15" t="s" s="70">
         <v>207</v>
       </c>
-      <c r="B15" t="s" s="65">
+      <c r="B15" t="s" s="70">
         <v>610</v>
       </c>
-      <c r="C15" t="s" s="65">
+      <c r="C15" t="s" s="70">
         <v>611</v>
       </c>
-      <c r="D15" t="s" s="65">
+      <c r="D15" t="s" s="70">
         <v>612</v>
       </c>
-      <c r="E15" s="66">
+      <c r="E15" s="72">
         <v>1</v>
       </c>
-      <c r="F15" t="s" s="65">
+      <c r="F15" t="s" s="70">
         <v>613</v>
       </c>
-      <c r="G15" t="s" s="65">
+      <c r="G15" t="s" s="70">
         <v>614</v>
       </c>
-      <c r="H15" t="s" s="65">
+      <c r="H15" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I15" s="30"/>
     </row>
     <row r="16" ht="19" customHeight="1">
-      <c r="A16" t="s" s="65">
+      <c r="A16" t="s" s="70">
         <v>215</v>
       </c>
-      <c r="B16" t="s" s="65">
+      <c r="B16" t="s" s="70">
         <v>615</v>
       </c>
-      <c r="C16" t="s" s="65">
+      <c r="C16" t="s" s="70">
         <v>616</v>
       </c>
-      <c r="D16" t="s" s="65">
+      <c r="D16" t="s" s="70">
         <v>617</v>
       </c>
-      <c r="E16" s="66">
+      <c r="E16" s="72">
         <v>1</v>
       </c>
-      <c r="F16" t="s" s="65">
+      <c r="F16" t="s" s="70">
         <v>618</v>
       </c>
-      <c r="G16" t="s" s="65">
+      <c r="G16" t="s" s="70">
         <v>619</v>
       </c>
-      <c r="H16" t="s" s="65">
+      <c r="H16" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I16" s="30"/>
     </row>
     <row r="17" ht="19" customHeight="1">
-      <c r="A17" t="s" s="65">
+      <c r="A17" t="s" s="70">
         <v>215</v>
       </c>
-      <c r="B17" t="s" s="65">
+      <c r="B17" t="s" s="70">
         <v>620</v>
       </c>
-      <c r="C17" t="s" s="65">
+      <c r="C17" t="s" s="70">
         <v>621</v>
       </c>
-      <c r="D17" t="s" s="65">
+      <c r="D17" t="s" s="70">
         <v>622</v>
       </c>
-      <c r="E17" s="66">
+      <c r="E17" s="72">
         <v>1</v>
       </c>
-      <c r="F17" t="s" s="65">
+      <c r="F17" t="s" s="70">
         <v>623</v>
       </c>
-      <c r="G17" t="s" s="65">
+      <c r="G17" t="s" s="70">
         <v>624</v>
       </c>
-      <c r="H17" t="s" s="65">
+      <c r="H17" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I17" s="30"/>
     </row>
     <row r="18" ht="19" customHeight="1">
-      <c r="A18" t="s" s="65">
+      <c r="A18" t="s" s="70">
         <v>215</v>
       </c>
-      <c r="B18" t="s" s="65">
+      <c r="B18" t="s" s="70">
         <v>625</v>
       </c>
-      <c r="C18" t="s" s="65">
+      <c r="C18" t="s" s="70">
         <v>626</v>
       </c>
-      <c r="D18" t="s" s="65">
+      <c r="D18" t="s" s="70">
         <v>627</v>
       </c>
-      <c r="E18" s="66">
+      <c r="E18" s="72">
         <v>2</v>
       </c>
-      <c r="F18" t="s" s="65">
+      <c r="F18" t="s" s="70">
         <v>628</v>
       </c>
-      <c r="G18" t="s" s="65">
+      <c r="G18" t="s" s="70">
         <v>629</v>
       </c>
-      <c r="H18" t="s" s="65">
+      <c r="H18" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I18" s="30"/>
     </row>
     <row r="19" ht="35" customHeight="1">
-      <c r="A19" t="s" s="65">
+      <c r="A19" t="s" s="70">
         <v>149</v>
       </c>
-      <c r="B19" t="s" s="65">
+      <c r="B19" t="s" s="70">
         <v>630</v>
       </c>
-      <c r="C19" t="s" s="65">
+      <c r="C19" t="s" s="70">
         <v>631</v>
       </c>
-      <c r="D19" t="s" s="65">
+      <c r="D19" t="s" s="70">
         <v>632</v>
       </c>
-      <c r="E19" s="66">
+      <c r="E19" s="72">
         <v>1</v>
       </c>
-      <c r="F19" t="s" s="65">
+      <c r="F19" t="s" s="70">
         <v>633</v>
       </c>
-      <c r="G19" t="s" s="65">
+      <c r="G19" t="s" s="70">
         <v>634</v>
       </c>
-      <c r="H19" t="s" s="65">
+      <c r="H19" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I19" s="30"/>
     </row>
     <row r="20" ht="35" customHeight="1">
-      <c r="A20" t="s" s="65">
+      <c r="A20" t="s" s="70">
         <v>149</v>
       </c>
-      <c r="B20" t="s" s="65">
+      <c r="B20" t="s" s="70">
         <v>635</v>
       </c>
-      <c r="C20" t="s" s="65">
+      <c r="C20" t="s" s="70">
         <v>636</v>
       </c>
-      <c r="D20" t="s" s="65">
+      <c r="D20" t="s" s="70">
         <v>637</v>
       </c>
-      <c r="E20" s="66">
+      <c r="E20" s="72">
         <v>1</v>
       </c>
-      <c r="F20" t="s" s="65">
+      <c r="F20" t="s" s="70">
         <v>638</v>
       </c>
-      <c r="G20" t="s" s="65">
+      <c r="G20" t="s" s="70">
         <v>639</v>
       </c>
-      <c r="H20" t="s" s="65">
+      <c r="H20" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I20" s="30"/>
     </row>
     <row r="21" ht="19" customHeight="1">
-      <c r="A21" t="s" s="65">
+      <c r="A21" t="s" s="70">
         <v>149</v>
       </c>
-      <c r="B21" t="s" s="65">
+      <c r="B21" t="s" s="70">
         <v>152</v>
       </c>
-      <c r="C21" t="s" s="65">
+      <c r="C21" t="s" s="70">
         <v>640</v>
       </c>
-      <c r="D21" t="s" s="65">
+      <c r="D21" t="s" s="70">
         <v>641</v>
       </c>
-      <c r="E21" s="66">
+      <c r="E21" s="72">
         <v>1</v>
       </c>
-      <c r="F21" t="s" s="65">
+      <c r="F21" t="s" s="70">
         <v>168</v>
       </c>
-      <c r="G21" t="s" s="65">
+      <c r="G21" t="s" s="70">
         <v>642</v>
       </c>
-      <c r="H21" t="s" s="65">
+      <c r="H21" t="s" s="70">
         <v>20</v>
       </c>
       <c r="I21" s="30"/>
     </row>
     <row r="22" ht="35" customHeight="1">
-      <c r="A22" t="s" s="65">
+      <c r="A22" t="s" s="70">
         <v>149</v>
       </c>
-      <c r="B22" t="s" s="65">
+      <c r="B22" t="s" s="70">
         <v>643</v>
       </c>
-      <c r="C22" t="s" s="65">
+      <c r="C22" t="s" s="70">
         <v>644</v>
       </c>
-      <c r="D22" t="s" s="65">
+      <c r="D22" t="s" s="70">
         <v>645</v>
       </c>
-      <c r="E22" s="66">
+      <c r="E22" s="72">
         <v>2</v>
       </c>
-      <c r="F22" t="s" s="65">
+      <c r="F22" t="s" s="70">
         <v>646</v>
       </c>
-      <c r="G22" t="s" s="65">
+      <c r="G22" t="s" s="70">
         <v>647</v>
       </c>
-      <c r="H22" t="s" s="65">
+      <c r="H22" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I22" s="30"/>
     </row>
     <row r="23" ht="19" customHeight="1">
-      <c r="A23" t="s" s="65">
+      <c r="A23" t="s" s="70">
         <v>231</v>
       </c>
-      <c r="B23" t="s" s="65">
+      <c r="B23" t="s" s="70">
         <v>648</v>
       </c>
-      <c r="C23" t="s" s="65">
+      <c r="C23" t="s" s="70">
         <v>649</v>
       </c>
-      <c r="D23" t="s" s="65">
+      <c r="D23" t="s" s="70">
         <v>650</v>
       </c>
-      <c r="E23" s="66">
+      <c r="E23" s="72">
         <v>1</v>
       </c>
-      <c r="F23" t="s" s="65">
+      <c r="F23" t="s" s="70">
         <v>651</v>
       </c>
-      <c r="G23" t="s" s="65">
+      <c r="G23" t="s" s="70">
         <v>652</v>
       </c>
-      <c r="H23" t="s" s="65">
+      <c r="H23" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I23" s="30"/>
     </row>
     <row r="24" ht="35" customHeight="1">
-      <c r="A24" t="s" s="65">
+      <c r="A24" t="s" s="70">
         <v>231</v>
       </c>
-      <c r="B24" t="s" s="65">
+      <c r="B24" t="s" s="70">
         <v>653</v>
       </c>
-      <c r="C24" t="s" s="65">
+      <c r="C24" t="s" s="70">
         <v>654</v>
       </c>
-      <c r="D24" t="s" s="65">
+      <c r="D24" t="s" s="70">
         <v>655</v>
       </c>
-      <c r="E24" s="66">
+      <c r="E24" s="72">
         <v>1</v>
       </c>
-      <c r="F24" t="s" s="65">
+      <c r="F24" t="s" s="70">
         <v>656</v>
       </c>
-      <c r="G24" t="s" s="65">
+      <c r="G24" t="s" s="70">
         <v>657</v>
       </c>
-      <c r="H24" t="s" s="65">
+      <c r="H24" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I24" s="30"/>
     </row>
     <row r="25" ht="35" customHeight="1">
-      <c r="A25" t="s" s="65">
+      <c r="A25" t="s" s="70">
         <v>239</v>
       </c>
-      <c r="B25" t="s" s="65">
+      <c r="B25" t="s" s="70">
         <v>658</v>
       </c>
-      <c r="C25" t="s" s="65">
+      <c r="C25" t="s" s="70">
         <v>659</v>
       </c>
-      <c r="D25" t="s" s="65">
+      <c r="D25" t="s" s="70">
         <v>660</v>
       </c>
-      <c r="E25" s="66">
+      <c r="E25" s="72">
         <v>1</v>
       </c>
-      <c r="F25" t="s" s="65">
+      <c r="F25" t="s" s="70">
         <v>661</v>
       </c>
-      <c r="G25" t="s" s="65">
+      <c r="G25" t="s" s="70">
         <v>662</v>
       </c>
-      <c r="H25" t="s" s="65">
+      <c r="H25" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I25" s="30"/>
     </row>
     <row r="26" ht="35" customHeight="1">
-      <c r="A26" t="s" s="65">
+      <c r="A26" t="s" s="70">
         <v>239</v>
       </c>
-      <c r="B26" t="s" s="65">
+      <c r="B26" t="s" s="70">
         <v>663</v>
       </c>
-      <c r="C26" t="s" s="65">
+      <c r="C26" t="s" s="70">
         <v>664</v>
       </c>
-      <c r="D26" t="s" s="65">
+      <c r="D26" t="s" s="70">
         <v>665</v>
       </c>
-      <c r="E26" s="66">
+      <c r="E26" s="72">
         <v>2</v>
       </c>
-      <c r="F26" t="s" s="65">
+      <c r="F26" t="s" s="70">
         <v>666</v>
       </c>
-      <c r="G26" t="s" s="65">
+      <c r="G26" t="s" s="70">
         <v>667</v>
       </c>
-      <c r="H26" t="s" s="65">
+      <c r="H26" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I26" s="30"/>
     </row>
     <row r="27" ht="35" customHeight="1">
-      <c r="A27" t="s" s="65">
+      <c r="A27" t="s" s="70">
         <v>247</v>
       </c>
-      <c r="B27" t="s" s="65">
+      <c r="B27" t="s" s="70">
         <v>668</v>
       </c>
-      <c r="C27" t="s" s="65">
+      <c r="C27" t="s" s="70">
         <v>669</v>
       </c>
-      <c r="D27" t="s" s="65">
+      <c r="D27" t="s" s="70">
         <v>670</v>
       </c>
-      <c r="E27" s="66">
+      <c r="E27" s="72">
         <v>1</v>
       </c>
-      <c r="F27" t="s" s="65">
+      <c r="F27" t="s" s="70">
         <v>671</v>
       </c>
-      <c r="G27" t="s" s="65">
+      <c r="G27" t="s" s="70">
         <v>672</v>
       </c>
-      <c r="H27" t="s" s="65">
+      <c r="H27" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I27" s="30"/>
     </row>
     <row r="28" ht="35" customHeight="1">
-      <c r="A28" t="s" s="65">
+      <c r="A28" t="s" s="70">
         <v>247</v>
       </c>
-      <c r="B28" t="s" s="65">
+      <c r="B28" t="s" s="70">
         <v>673</v>
       </c>
-      <c r="C28" t="s" s="65">
+      <c r="C28" t="s" s="70">
         <v>674</v>
       </c>
-      <c r="D28" t="s" s="65">
+      <c r="D28" t="s" s="70">
         <v>675</v>
       </c>
-      <c r="E28" s="66">
+      <c r="E28" s="72">
         <v>2</v>
       </c>
-      <c r="F28" t="s" s="65">
+      <c r="F28" t="s" s="70">
         <v>676</v>
       </c>
-      <c r="G28" t="s" s="65">
+      <c r="G28" t="s" s="70">
         <v>677</v>
       </c>
-      <c r="H28" t="s" s="65">
+      <c r="H28" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I28" s="30"/>
     </row>
     <row r="29" ht="35" customHeight="1">
-      <c r="A29" t="s" s="65">
+      <c r="A29" t="s" s="70">
         <v>255</v>
       </c>
-      <c r="B29" t="s" s="65">
+      <c r="B29" t="s" s="70">
         <v>678</v>
       </c>
-      <c r="C29" t="s" s="65">
+      <c r="C29" t="s" s="70">
         <v>679</v>
       </c>
-      <c r="D29" t="s" s="65">
+      <c r="D29" t="s" s="70">
         <v>680</v>
       </c>
-      <c r="E29" s="66">
+      <c r="E29" s="72">
         <v>1</v>
       </c>
-      <c r="F29" t="s" s="65">
+      <c r="F29" t="s" s="70">
         <v>681</v>
       </c>
-      <c r="G29" t="s" s="65">
+      <c r="G29" t="s" s="70">
         <v>682</v>
       </c>
-      <c r="H29" t="s" s="65">
+      <c r="H29" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I29" s="30"/>
     </row>
     <row r="30" ht="35" customHeight="1">
-      <c r="A30" t="s" s="65">
+      <c r="A30" t="s" s="70">
         <v>255</v>
       </c>
-      <c r="B30" t="s" s="65">
+      <c r="B30" t="s" s="70">
         <v>683</v>
       </c>
-      <c r="C30" t="s" s="65">
+      <c r="C30" t="s" s="70">
         <v>684</v>
       </c>
-      <c r="D30" t="s" s="65">
+      <c r="D30" t="s" s="70">
         <v>685</v>
       </c>
-      <c r="E30" s="66">
+      <c r="E30" s="72">
         <v>2</v>
       </c>
-      <c r="F30" t="s" s="65">
+      <c r="F30" t="s" s="70">
         <v>686</v>
       </c>
-      <c r="G30" t="s" s="65">
+      <c r="G30" t="s" s="70">
         <v>687</v>
       </c>
-      <c r="H30" t="s" s="65">
+      <c r="H30" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I30" s="30"/>
     </row>
     <row r="31" ht="37.4" customHeight="1">
-      <c r="A31" t="s" s="65">
+      <c r="A31" t="s" s="70">
         <v>263</v>
       </c>
-      <c r="B31" t="s" s="65">
+      <c r="B31" t="s" s="70">
         <v>688</v>
       </c>
-      <c r="C31" t="s" s="65">
+      <c r="C31" t="s" s="70">
         <v>689</v>
       </c>
-      <c r="D31" t="s" s="65">
+      <c r="D31" t="s" s="70">
         <v>690</v>
       </c>
-      <c r="E31" s="66">
+      <c r="E31" s="72">
         <v>1</v>
       </c>
-      <c r="F31" t="s" s="65">
+      <c r="F31" t="s" s="70">
         <v>691</v>
       </c>
-      <c r="G31" t="s" s="65">
+      <c r="G31" t="s" s="70">
         <v>619</v>
       </c>
-      <c r="H31" t="s" s="65">
+      <c r="H31" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I31" s="30"/>
     </row>
     <row r="32" ht="35" customHeight="1">
-      <c r="A32" t="s" s="65">
+      <c r="A32" t="s" s="70">
         <v>263</v>
       </c>
-      <c r="B32" t="s" s="65">
+      <c r="B32" t="s" s="70">
         <v>692</v>
       </c>
-      <c r="C32" t="s" s="65">
+      <c r="C32" t="s" s="70">
         <v>693</v>
       </c>
-      <c r="D32" t="s" s="65">
+      <c r="D32" t="s" s="70">
         <v>694</v>
       </c>
-      <c r="E32" s="66">
+      <c r="E32" s="72">
         <v>1</v>
       </c>
-      <c r="F32" t="s" s="65">
+      <c r="F32" t="s" s="70">
         <v>695</v>
       </c>
-      <c r="G32" t="s" s="65">
+      <c r="G32" t="s" s="70">
         <v>696</v>
       </c>
-      <c r="H32" t="s" s="65">
+      <c r="H32" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I32" s="30"/>
     </row>
     <row r="33" ht="35" customHeight="1">
-      <c r="A33" t="s" s="65">
+      <c r="A33" t="s" s="70">
         <v>263</v>
       </c>
-      <c r="B33" t="s" s="65">
+      <c r="B33" t="s" s="70">
         <v>697</v>
       </c>
-      <c r="C33" t="s" s="65">
+      <c r="C33" t="s" s="70">
         <v>698</v>
       </c>
-      <c r="D33" t="s" s="65">
+      <c r="D33" t="s" s="70">
         <v>699</v>
       </c>
-      <c r="E33" s="66">
+      <c r="E33" s="72">
         <v>1</v>
       </c>
-      <c r="F33" t="s" s="65">
+      <c r="F33" t="s" s="70">
         <v>700</v>
       </c>
-      <c r="G33" t="s" s="65">
+      <c r="G33" t="s" s="70">
         <v>701</v>
       </c>
-      <c r="H33" t="s" s="65">
+      <c r="H33" t="s" s="70">
         <v>295</v>
       </c>
       <c r="I33" s="30"/>
     </row>
     <row r="34" ht="35" customHeight="1">
-      <c r="A34" t="s" s="73">
+      <c r="A34" t="s" s="79">
         <v>271</v>
       </c>
-      <c r="B34" t="s" s="65">
+      <c r="B34" t="s" s="70">
         <v>702</v>
       </c>
-      <c r="C34" t="s" s="65">
+      <c r="C34" t="s" s="70">
         <v>703</v>
       </c>
-      <c r="D34" t="s" s="65">
+      <c r="D34" t="s" s="70">
         <v>704</v>
       </c>
-      <c r="E34" s="66">
+      <c r="E34" s="72">
         <v>1</v>
       </c>
-      <c r="F34" t="s" s="65">
+      <c r="F34" t="s" s="70">
         <v>705</v>
       </c>
-      <c r="G34" t="s" s="65">
+      <c r="G34" t="s" s="70">
         <v>706</v>
       </c>
-      <c r="H34" s="74"/>
+      <c r="H34" s="80"/>
       <c r="I34" s="29"/>
     </row>
     <row r="35" ht="35" customHeight="1">
-      <c r="A35" t="s" s="73">
+      <c r="A35" t="s" s="79">
         <v>271</v>
       </c>
-      <c r="B35" t="s" s="65">
+      <c r="B35" t="s" s="70">
         <v>707</v>
       </c>
-      <c r="C35" t="s" s="65">
+      <c r="C35" t="s" s="70">
         <v>708</v>
       </c>
-      <c r="D35" t="s" s="65">
+      <c r="D35" t="s" s="70">
         <v>709</v>
       </c>
-      <c r="E35" s="66">
+      <c r="E35" s="72">
         <v>1</v>
       </c>
-      <c r="F35" t="s" s="65">
+      <c r="F35" t="s" s="70">
         <v>710</v>
       </c>
-      <c r="G35" t="s" s="65">
+      <c r="G35" t="s" s="70">
         <v>711</v>
       </c>
-      <c r="H35" s="74"/>
+      <c r="H35" s="80"/>
       <c r="I35" s="29"/>
     </row>
     <row r="36" ht="35" customHeight="1">
-      <c r="A36" t="s" s="73">
+      <c r="A36" t="s" s="79">
         <v>271</v>
       </c>
-      <c r="B36" t="s" s="65">
+      <c r="B36" t="s" s="70">
         <v>712</v>
       </c>
-      <c r="C36" t="s" s="65">
+      <c r="C36" t="s" s="70">
         <v>713</v>
       </c>
-      <c r="D36" t="s" s="65">
+      <c r="D36" t="s" s="70">
         <v>714</v>
       </c>
-      <c r="E36" s="66">
+      <c r="E36" s="72">
         <v>2</v>
       </c>
-      <c r="F36" t="s" s="65">
+      <c r="F36" t="s" s="70">
         <v>715</v>
       </c>
-      <c r="G36" t="s" s="65">
+      <c r="G36" t="s" s="70">
         <v>589</v>
       </c>
-      <c r="H36" s="74"/>
+      <c r="H36" s="80"/>
       <c r="I36" s="29"/>
     </row>
     <row r="37" ht="53.4" customHeight="1">
-      <c r="A37" t="s" s="73">
+      <c r="A37" t="s" s="79">
         <v>280</v>
       </c>
-      <c r="B37" t="s" s="65">
+      <c r="B37" t="s" s="70">
         <v>716</v>
       </c>
-      <c r="C37" t="s" s="65">
+      <c r="C37" t="s" s="70">
         <v>717</v>
       </c>
-      <c r="D37" t="s" s="65">
+      <c r="D37" t="s" s="70">
         <v>718</v>
       </c>
-      <c r="E37" s="66">
+      <c r="E37" s="72">
         <v>1</v>
       </c>
-      <c r="F37" t="s" s="65">
+      <c r="F37" t="s" s="70">
         <v>719</v>
       </c>
-      <c r="G37" t="s" s="65">
+      <c r="G37" t="s" s="70">
         <v>720</v>
       </c>
-      <c r="H37" s="74"/>
+      <c r="H37" s="80"/>
       <c r="I37" s="29"/>
     </row>
     <row r="38" ht="35" customHeight="1">
-      <c r="A38" t="s" s="73">
+      <c r="A38" t="s" s="79">
         <v>280</v>
       </c>
-      <c r="B38" t="s" s="65">
+      <c r="B38" t="s" s="70">
         <v>721</v>
       </c>
-      <c r="C38" t="s" s="65">
+      <c r="C38" t="s" s="70">
         <v>722</v>
       </c>
-      <c r="D38" t="s" s="65">
+      <c r="D38" t="s" s="70">
         <v>723</v>
       </c>
-      <c r="E38" s="66">
+      <c r="E38" s="72">
         <v>2</v>
       </c>
-      <c r="F38" t="s" s="65">
+      <c r="F38" t="s" s="70">
         <v>724</v>
       </c>
-      <c r="G38" t="s" s="65">
+      <c r="G38" t="s" s="70">
         <v>725</v>
       </c>
-      <c r="H38" s="74"/>
+      <c r="H38" s="80"/>
       <c r="I38" s="29"/>
-    </row>
-    <row r="39" ht="15" customHeight="1">
-      <c r="A39" t="s" s="90">
-        <v>33</v>
-      </c>
-      <c r="B39" t="s" s="91">
-        <v>726</v>
-      </c>
-      <c r="C39" t="s" s="91">
-        <v>727</v>
-      </c>
-      <c r="D39" t="s" s="91">
-        <v>728</v>
-      </c>
-      <c r="E39" s="92">
-        <v>1</v>
-      </c>
-      <c r="F39" t="s" s="91">
-        <v>729</v>
-      </c>
-      <c r="G39" t="s" s="91">
-        <v>730</v>
-      </c>
-      <c r="H39" s="93"/>
-      <c r="I39" s="94"/>
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -9524,10 +9492,10 @@
   <dimension ref="A1:H11"/>
   <sheetFormatPr defaultColWidth="8.83333" defaultRowHeight="15" customHeight="1" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col min="1" max="1" width="20" style="95" customWidth="1"/>
-    <col min="2" max="2" width="100" style="95" customWidth="1"/>
-    <col min="3" max="8" width="8.85156" style="95" customWidth="1"/>
-    <col min="9" max="16384" width="8.85156" style="95" customWidth="1"/>
+    <col min="1" max="1" width="20" style="97" customWidth="1"/>
+    <col min="2" max="2" width="100" style="97" customWidth="1"/>
+    <col min="3" max="8" width="8.85156" style="97" customWidth="1"/>
+    <col min="9" max="16384" width="8.85156" style="97" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" ht="25.5" customHeight="1">
@@ -9544,7 +9512,7 @@
     </row>
     <row r="2" ht="25.5" customHeight="1">
       <c r="A2" t="s" s="5">
-        <v>731</v>
+        <v>726</v>
       </c>
       <c r="B2" s="6"/>
       <c r="C2" s="6"/>
@@ -9580,10 +9548,10 @@
     </row>
     <row r="5" ht="26.55" customHeight="1">
       <c r="A5" t="s" s="31">
-        <v>732</v>
+        <v>727</v>
       </c>
       <c r="B5" t="s" s="33">
-        <v>733</v>
+        <v>728</v>
       </c>
       <c r="C5" s="12"/>
       <c r="D5" s="13"/>
@@ -9597,7 +9565,7 @@
         <v>10</v>
       </c>
       <c r="B6" t="s" s="36">
-        <v>734</v>
+        <v>729</v>
       </c>
       <c r="C6" s="12"/>
       <c r="D6" s="13"/>
@@ -9611,7 +9579,7 @@
         <v>79</v>
       </c>
       <c r="B7" t="s" s="33">
-        <v>735</v>
+        <v>730</v>
       </c>
       <c r="C7" s="12"/>
       <c r="D7" s="13"/>
@@ -9625,7 +9593,7 @@
         <v>162</v>
       </c>
       <c r="B8" t="s" s="36">
-        <v>735</v>
+        <v>730</v>
       </c>
       <c r="C8" s="12"/>
       <c r="D8" s="13"/>
@@ -9639,7 +9607,7 @@
         <v>127</v>
       </c>
       <c r="B9" t="s" s="33">
-        <v>736</v>
+        <v>731</v>
       </c>
       <c r="C9" s="12"/>
       <c r="D9" s="13"/>
@@ -9649,11 +9617,11 @@
       <c r="H9" s="13"/>
     </row>
     <row r="10" ht="13.55" customHeight="1">
-      <c r="A10" t="s" s="85">
-        <v>737</v>
-      </c>
-      <c r="B10" t="s" s="88">
-        <v>738</v>
+      <c r="A10" t="s" s="92">
+        <v>732</v>
+      </c>
+      <c r="B10" t="s" s="95">
+        <v>733</v>
       </c>
       <c r="C10" s="12"/>
       <c r="D10" s="13"/>
@@ -9663,8 +9631,8 @@
       <c r="H10" s="13"/>
     </row>
     <row r="11" ht="13.55" customHeight="1">
-      <c r="A11" s="96"/>
-      <c r="B11" s="96"/>
+      <c r="A11" s="98"/>
+      <c r="B11" s="98"/>
       <c r="C11" s="13"/>
       <c r="D11" s="13"/>
       <c r="E11" s="13"/>

</xml_diff>